<commit_message>
Added psi to TCC
</commit_message>
<xml_diff>
--- a/Database/260126_Datenbankdefinition.xlsx
+++ b/Database/260126_Datenbankdefinition.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jonathanbieg/Documents/Master Thesis/1_Code/Python Repository/SDSD_Bieg/Database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31C98FBF-6703-D746-A4D1-D8677F03FC07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2763DDFA-6CF9-BD46-A06B-41F25BD259C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14840" yWindow="840" windowWidth="14360" windowHeight="16700" firstSheet="1" activeTab="1" xr2:uid="{58B6788A-438B-478E-898A-D53025B55ED1}"/>
+    <workbookView xWindow="14840" yWindow="840" windowWidth="14360" windowHeight="16700" activeTab="3" xr2:uid="{58B6788A-438B-478E-898A-D53025B55ED1}"/>
   </bookViews>
   <sheets>
     <sheet name="products" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Created Database with phi and connector_TCC, created simple_span_1d_TCC(Test260311)
</commit_message>
<xml_diff>
--- a/Database/260126_Datenbankdefinition.xlsx
+++ b/Database/260126_Datenbankdefinition.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jonathanbieg/Documents/Master Thesis/1_Code/Python Repository/SDSD_Bieg/Database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2763DDFA-6CF9-BD46-A06B-41F25BD259C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46CB7A72-0FDC-CB47-B4C6-92AD6D2553C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14840" yWindow="840" windowWidth="14360" windowHeight="16700" activeTab="3" xr2:uid="{58B6788A-438B-478E-898A-D53025B55ED1}"/>
+    <workbookView xWindow="14840" yWindow="840" windowWidth="15420" windowHeight="16700" activeTab="1" xr2:uid="{58B6788A-438B-478E-898A-D53025B55ED1}"/>
   </bookViews>
   <sheets>
     <sheet name="products" sheetId="1" r:id="rId1"/>
@@ -2770,216 +2770,6 @@
         <bottom style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4"/>
-          <bgColor theme="4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -3971,6 +3761,216 @@
       </font>
       <alignment vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -4041,42 +4041,42 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{690E7B34-75E3-43BA-8CDD-44A4EFCCEFD5}" name="Table2" displayName="Table2" ref="A1:AB132" totalsRowShown="0" headerRowDxfId="55" dataDxfId="54">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{690E7B34-75E3-43BA-8CDD-44A4EFCCEFD5}" name="Table2" displayName="Table2" ref="A1:AB132" totalsRowShown="0" headerRowDxfId="46" dataDxfId="45">
   <autoFilter ref="A1:AB132" xr:uid="{690E7B34-75E3-43BA-8CDD-44A4EFCCEFD5}"/>
   <tableColumns count="28">
-    <tableColumn id="9" xr3:uid="{1DBBD25D-72F9-4A81-9CFA-500505E3628D}" name="ID" dataDxfId="53"/>
-    <tableColumn id="14" xr3:uid="{6844A52F-C967-44C0-BF5C-160C47AB6E64}" name="PRO_ID" dataDxfId="52"/>
-    <tableColumn id="12" xr3:uid="{4EDF1E73-4744-474F-8DFE-7F72FB05613C}" name="EPD_ID" dataDxfId="51"/>
-    <tableColumn id="1" xr3:uid="{1CF2E22E-1020-4F35-B31F-6350A15A5DE8}" name="SOURCE" dataDxfId="50"/>
-    <tableColumn id="27" xr3:uid="{07F74D5D-9130-4120-B02C-A11234427F46}" name="KBOB ID-Nr." dataDxfId="49"/>
-    <tableColumn id="11" xr3:uid="{81FE7F31-5F54-40F9-B99E-827E048F7DB5}" name="EPD_DATE" dataDxfId="48"/>
-    <tableColumn id="10" xr3:uid="{54D8BA04-0FEF-4C3B-9B14-59E8F982CD3F}" name="VALID_TO" dataDxfId="47"/>
-    <tableColumn id="22" xr3:uid="{3D6FC370-B8A8-40C3-9FC8-791B178DDFDF}" name="COUNTRY" dataDxfId="46"/>
-    <tableColumn id="4" xr3:uid="{25C7280F-4E3E-4E39-BDBB-DC06DF090C5B}" name="PRODUCT_NAME" dataDxfId="45"/>
-    <tableColumn id="26" xr3:uid="{1053A7DD-B11F-4E75-92EC-BC0F866E90B4}" name="OEKOBAUDAT_ID" dataDxfId="44"/>
-    <tableColumn id="25" xr3:uid="{295F99F8-E318-45C9-833E-F0B45A26471A}" name="MATERIAL_GROUP" dataDxfId="43"/>
-    <tableColumn id="2" xr3:uid="{1326FCEF-D1EE-4F3A-BB8B-77CB4EC72B0C}" name="MATERIAL" dataDxfId="42"/>
-    <tableColumn id="5" xr3:uid="{9B2A7F84-D968-4A00-B61F-23BB0661E7A3}" name="CEMENT" dataDxfId="41"/>
-    <tableColumn id="6" xr3:uid="{2F6E5831-6238-4360-9CFD-ED23A193E761}" name="MECH_PROP" dataDxfId="40"/>
-    <tableColumn id="13" xr3:uid="{50DAB01C-8AF5-4E0C-9904-54F70B81BC55}" name="DENSITY" dataDxfId="39"/>
-    <tableColumn id="18" xr3:uid="{F799A4D4-9543-475F-989E-CFBA47249558}" name="EXPOSITIONSKLASSE" dataDxfId="38"/>
-    <tableColumn id="17" xr3:uid="{ECCBC067-991C-4C60-942D-806BCD77B990}" name="GROESSTKORN" dataDxfId="37"/>
-    <tableColumn id="16" xr3:uid="{05157B85-D5FB-4844-9B53-D8AB09BCE0D9}" name="CHLORIDGEHALT" dataDxfId="36"/>
-    <tableColumn id="15" xr3:uid="{9F53CF50-7148-405A-9295-1F0C3C45645A}" name="KONSISTENZKLASSE" dataDxfId="35"/>
-    <tableColumn id="7" xr3:uid="{E23232F6-E86E-4AD2-8257-F30C0D1F7368}" name="Total_GWP" dataDxfId="34"/>
-    <tableColumn id="20" xr3:uid="{0A9001B4-3AB4-4C58-B125-0B2AA4DB2681}" name="A1toA3_GWP" dataDxfId="33">
+    <tableColumn id="9" xr3:uid="{1DBBD25D-72F9-4A81-9CFA-500505E3628D}" name="ID" dataDxfId="44"/>
+    <tableColumn id="14" xr3:uid="{6844A52F-C967-44C0-BF5C-160C47AB6E64}" name="PRO_ID" dataDxfId="43"/>
+    <tableColumn id="12" xr3:uid="{4EDF1E73-4744-474F-8DFE-7F72FB05613C}" name="EPD_ID" dataDxfId="42"/>
+    <tableColumn id="1" xr3:uid="{1CF2E22E-1020-4F35-B31F-6350A15A5DE8}" name="SOURCE" dataDxfId="41"/>
+    <tableColumn id="27" xr3:uid="{07F74D5D-9130-4120-B02C-A11234427F46}" name="KBOB ID-Nr." dataDxfId="40"/>
+    <tableColumn id="11" xr3:uid="{81FE7F31-5F54-40F9-B99E-827E048F7DB5}" name="EPD_DATE" dataDxfId="39"/>
+    <tableColumn id="10" xr3:uid="{54D8BA04-0FEF-4C3B-9B14-59E8F982CD3F}" name="VALID_TO" dataDxfId="38"/>
+    <tableColumn id="22" xr3:uid="{3D6FC370-B8A8-40C3-9FC8-791B178DDFDF}" name="COUNTRY" dataDxfId="37"/>
+    <tableColumn id="4" xr3:uid="{25C7280F-4E3E-4E39-BDBB-DC06DF090C5B}" name="PRODUCT_NAME" dataDxfId="36"/>
+    <tableColumn id="26" xr3:uid="{1053A7DD-B11F-4E75-92EC-BC0F866E90B4}" name="OEKOBAUDAT_ID" dataDxfId="35"/>
+    <tableColumn id="25" xr3:uid="{295F99F8-E318-45C9-833E-F0B45A26471A}" name="MATERIAL_GROUP" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{1326FCEF-D1EE-4F3A-BB8B-77CB4EC72B0C}" name="MATERIAL" dataDxfId="33"/>
+    <tableColumn id="5" xr3:uid="{9B2A7F84-D968-4A00-B61F-23BB0661E7A3}" name="CEMENT" dataDxfId="32"/>
+    <tableColumn id="6" xr3:uid="{2F6E5831-6238-4360-9CFD-ED23A193E761}" name="MECH_PROP" dataDxfId="31"/>
+    <tableColumn id="13" xr3:uid="{50DAB01C-8AF5-4E0C-9904-54F70B81BC55}" name="DENSITY" dataDxfId="30"/>
+    <tableColumn id="18" xr3:uid="{F799A4D4-9543-475F-989E-CFBA47249558}" name="EXPOSITIONSKLASSE" dataDxfId="29"/>
+    <tableColumn id="17" xr3:uid="{ECCBC067-991C-4C60-942D-806BCD77B990}" name="GROESSTKORN" dataDxfId="28"/>
+    <tableColumn id="16" xr3:uid="{05157B85-D5FB-4844-9B53-D8AB09BCE0D9}" name="CHLORIDGEHALT" dataDxfId="27"/>
+    <tableColumn id="15" xr3:uid="{9F53CF50-7148-405A-9295-1F0C3C45645A}" name="KONSISTENZKLASSE" dataDxfId="26"/>
+    <tableColumn id="7" xr3:uid="{E23232F6-E86E-4AD2-8257-F30C0D1F7368}" name="Total_GWP" dataDxfId="25"/>
+    <tableColumn id="20" xr3:uid="{0A9001B4-3AB4-4C58-B125-0B2AA4DB2681}" name="A1toA3_GWP" dataDxfId="24">
       <calculatedColumnFormula>119+10.9+238</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="21" xr3:uid="{2799394A-C481-45CE-B194-AAABAB0AED38}" name="C1toC4_GWP" dataDxfId="32">
+    <tableColumn id="21" xr3:uid="{2799394A-C481-45CE-B194-AAABAB0AED38}" name="C1toC4_GWP" dataDxfId="23">
       <calculatedColumnFormula>51.1+26+2.64+12.6</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="19" xr3:uid="{70561D70-9D02-4E93-A395-229DA8696DDA}" name="ValidEPD" dataDxfId="31">
+    <tableColumn id="19" xr3:uid="{70561D70-9D02-4E93-A395-229DA8696DDA}" name="ValidEPD" dataDxfId="22">
       <calculatedColumnFormula>IF(OR($D2="Ecoinvent",$D2="Betonsortenrechner",$D2="KBOB",$T2&lt;=0),0,1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="29" xr3:uid="{92D55BC7-F55B-406A-B127-69EC2F0A8B77}" name="noch gültig" dataDxfId="30">
+    <tableColumn id="29" xr3:uid="{92D55BC7-F55B-406A-B127-69EC2F0A8B77}" name="noch gültig" dataDxfId="21">
       <calculatedColumnFormula>IF(Table2[[#This Row],[VALID_TO]]&gt;=TODAY(), 1, 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{DB90AC0A-8933-4040-BADE-E6EE11AC8BD7}" name="Statistik" dataDxfId="29">
+    <tableColumn id="3" xr3:uid="{DB90AC0A-8933-4040-BADE-E6EE11AC8BD7}" name="Statistik" dataDxfId="20">
       <calculatedColumnFormula array="1">IF($W2&lt;&gt;0,
 IF(AND(
                          T2&gt;=_xlfn.PERCENTILE.INC(_xlfn._xlws.FILTER($T$2:$T$148, ($L$2:$L$148=L2)*($W$2:$W$148=1)),0.1),
@@ -4084,41 +4084,41 @@
                ),1,0),
 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{BBA6C134-63F9-4711-8B25-086098EC2CB0}" name="Cost" dataDxfId="28"/>
-    <tableColumn id="24" xr3:uid="{5321A0E1-043C-4E95-A6DA-41830364B2BC}" name="Anmerkung" dataDxfId="27"/>
-    <tableColumn id="23" xr3:uid="{61456234-34E8-4222-B2D6-9DDA8E83B081}" name="Spalte 1" dataDxfId="26"/>
+    <tableColumn id="8" xr3:uid="{BBA6C134-63F9-4711-8B25-086098EC2CB0}" name="Cost" dataDxfId="19"/>
+    <tableColumn id="24" xr3:uid="{5321A0E1-043C-4E95-A6DA-41830364B2BC}" name="Anmerkung" dataDxfId="18"/>
+    <tableColumn id="23" xr3:uid="{61456234-34E8-4222-B2D6-9DDA8E83B081}" name="Spalte 1" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{188FAA96-3B75-4826-B66B-A81D5BCFC670}" name="Tabelle4" displayName="Tabelle4" ref="A1:J8" totalsRowShown="0" headerRowDxfId="25" dataDxfId="23" headerRowBorderDxfId="24" tableBorderDxfId="22" totalsRowBorderDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{188FAA96-3B75-4826-B66B-A81D5BCFC670}" name="Tabelle4" displayName="Tabelle4" ref="A1:J8" totalsRowShown="0" headerRowDxfId="16" dataDxfId="14" headerRowBorderDxfId="15" tableBorderDxfId="13" totalsRowBorderDxfId="12">
   <autoFilter ref="A1:J8" xr:uid="{188FAA96-3B75-4826-B66B-A81D5BCFC670}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{AF3C694B-2C8A-40EE-B8BB-2EC9EB81A87A}" name="mat_ID" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{B447FBC2-C455-4332-8F47-150B112A57E0}" name="name" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{BAFC6B47-7268-46CC-A881-892C9A1F4334}" name="strength_comp" dataDxfId="18"/>
-    <tableColumn id="4" xr3:uid="{6FC4C8EB-7581-4E67-81CE-C724161F0838}" name="strength_tens" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{A875970E-61A9-43B5-9361-7616A74C3147}" name="strength_bend" dataDxfId="16"/>
-    <tableColumn id="6" xr3:uid="{EF5B3A69-DD70-420A-88FF-4FE8772A2E14}" name="strength_shea" dataDxfId="15"/>
-    <tableColumn id="7" xr3:uid="{ED461A80-736C-42BD-81BC-C5C0C80FF34C}" name="E_modulus" dataDxfId="14"/>
-    <tableColumn id="8" xr3:uid="{68E47481-7028-4427-B126-2A046FC46737}" name="density_load" dataDxfId="13"/>
-    <tableColumn id="9" xr3:uid="{7AB34570-2BD4-417F-B141-70612577C7D6}" name="burn_rate" dataDxfId="12"/>
-    <tableColumn id="10" xr3:uid="{69298654-E280-9D4B-9717-7904FADC15B5}" name="phi" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{AF3C694B-2C8A-40EE-B8BB-2EC9EB81A87A}" name="mat_ID" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{B447FBC2-C455-4332-8F47-150B112A57E0}" name="name" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{BAFC6B47-7268-46CC-A881-892C9A1F4334}" name="strength_comp" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{6FC4C8EB-7581-4E67-81CE-C724161F0838}" name="strength_tens" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{A875970E-61A9-43B5-9361-7616A74C3147}" name="strength_bend" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{EF5B3A69-DD70-420A-88FF-4FE8772A2E14}" name="strength_shea" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{ED461A80-736C-42BD-81BC-C5C0C80FF34C}" name="E_modulus" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{68E47481-7028-4427-B126-2A046FC46737}" name="density_load" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{7AB34570-2BD4-417F-B141-70612577C7D6}" name="burn_rate" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{69298654-E280-9D4B-9717-7904FADC15B5}" name="phi" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1CD264FD-E2C0-E94F-B387-736226CC982D}" name="Tabelle42" displayName="Tabelle42" ref="A1:D6" totalsRowShown="0" headerRowDxfId="10" dataDxfId="8" headerRowBorderDxfId="9" tableBorderDxfId="7" totalsRowBorderDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1CD264FD-E2C0-E94F-B387-736226CC982D}" name="Tabelle42" displayName="Tabelle42" ref="A1:D6" totalsRowShown="0" headerRowDxfId="55" dataDxfId="53" headerRowBorderDxfId="54" tableBorderDxfId="52" totalsRowBorderDxfId="51">
   <autoFilter ref="A1:D6" xr:uid="{1CD264FD-E2C0-E94F-B387-736226CC982D}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{6590463D-C242-4C4D-AA1F-6FA1F0D35E6F}" name="mat_ID" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{603BAED4-55F2-D040-9D73-1611C1564A84}" name="name" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{D6CC67C0-1ACA-D446-A6F3-00BCC3AC8DAC}" name="d [m]" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{3D62C7FF-3D7F-B245-A874-3A95DF0C49D2}" name="K_ser [N/m]2" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{6590463D-C242-4C4D-AA1F-6FA1F0D35E6F}" name="mat_ID" dataDxfId="50"/>
+    <tableColumn id="2" xr3:uid="{603BAED4-55F2-D040-9D73-1611C1564A84}" name="name" dataDxfId="49"/>
+    <tableColumn id="3" xr3:uid="{D6CC67C0-1ACA-D446-A6F3-00BCC3AC8DAC}" name="d [m]" dataDxfId="48"/>
+    <tableColumn id="4" xr3:uid="{3D62C7FF-3D7F-B245-A874-3A95DF0C49D2}" name="K_ser [N/m]2" dataDxfId="47"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>

</xml_diff>

<commit_message>
Able now to plot TCC, seems wrong.
</commit_message>
<xml_diff>
--- a/Database/260126_Datenbankdefinition.xlsx
+++ b/Database/260126_Datenbankdefinition.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jonathanbieg/Documents/Master Thesis/1_Code/Python Repository/SDSD_Bieg/Database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CD6F826-6D3D-4644-8BD7-775F45A8B808}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{867534AF-8429-4447-B406-3AA3D1D176DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13980" yWindow="840" windowWidth="15420" windowHeight="16700" activeTab="3" xr2:uid="{58B6788A-438B-478E-898A-D53025B55ED1}"/>
+    <workbookView xWindow="600" yWindow="840" windowWidth="25180" windowHeight="16700" activeTab="3" xr2:uid="{58B6788A-438B-478E-898A-D53025B55ED1}"/>
   </bookViews>
   <sheets>
     <sheet name="products" sheetId="1" r:id="rId1"/>
@@ -1663,16 +1663,16 @@
     <t>DBS_12</t>
   </si>
   <si>
-    <t>d [m]</t>
-  </si>
-  <si>
     <t>phi</t>
   </si>
   <si>
-    <t>K_ser [N/m]</t>
-  </si>
-  <si>
     <t>kerve</t>
+  </si>
+  <si>
+    <t>K_ser</t>
+  </si>
+  <si>
+    <t>d</t>
   </si>
 </sst>
 </file>
@@ -3579,7 +3579,7 @@
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor auto="1"/>
+          <bgColor indexed="65"/>
         </patternFill>
       </fill>
       <border diagonalUp="0" diagonalDown="0">
@@ -3591,6 +3591,8 @@
         <bottom style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </bottom>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -3613,10 +3615,10 @@
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor auto="1"/>
+          <bgColor indexed="65"/>
         </patternFill>
       </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
+      <border diagonalUp="0" diagonalDown="0">
         <left/>
         <right/>
         <top style="thin">
@@ -3625,6 +3627,8 @@
         <bottom style="thin">
           <color theme="4" tint="0.39997558519241921"/>
         </bottom>
+        <vertical/>
+        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -4117,8 +4121,8 @@
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{6590463D-C242-4C4D-AA1F-6FA1F0D35E6F}" name="mat_ID" dataDxfId="5"/>
     <tableColumn id="2" xr3:uid="{603BAED4-55F2-D040-9D73-1611C1564A84}" name="name" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{D6CC67C0-1ACA-D446-A6F3-00BCC3AC8DAC}" name="d [m]" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{3D62C7FF-3D7F-B245-A874-3A95DF0C49D2}" name="K_ser [N/m]" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{D6CC67C0-1ACA-D446-A6F3-00BCC3AC8DAC}" name="d" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{3D62C7FF-3D7F-B245-A874-3A95DF0C49D2}" name="K_ser" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -15987,7 +15991,7 @@
         <v>414</v>
       </c>
       <c r="J1" s="61" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
@@ -16363,7 +16367,7 @@
         <v>407</v>
       </c>
       <c r="C1" s="61" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="D1" s="61" t="s">
         <v>519</v>
@@ -16430,7 +16434,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="56" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="C6" s="56"/>
       <c r="D6" s="56">

</xml_diff>

<commit_message>
Fixed vu of TCC
</commit_message>
<xml_diff>
--- a/Database/260126_Datenbankdefinition.xlsx
+++ b/Database/260126_Datenbankdefinition.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jonathanbieg/Documents/Master Thesis/1_Code/Python Repository/SDSD_Bieg/Database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{867534AF-8429-4447-B406-3AA3D1D176DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BFD5328-3A24-ED40-B0B1-D0BD7F14B997}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="600" yWindow="840" windowWidth="25180" windowHeight="16700" activeTab="3" xr2:uid="{58B6788A-438B-478E-898A-D53025B55ED1}"/>
+    <workbookView xWindow="600" yWindow="840" windowWidth="25180" windowHeight="16700" activeTab="2" xr2:uid="{58B6788A-438B-478E-898A-D53025B55ED1}"/>
   </bookViews>
   <sheets>
     <sheet name="products" sheetId="1" r:id="rId1"/>
@@ -2758,7 +2758,7 @@
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor auto="1"/>
+          <bgColor indexed="65"/>
         </patternFill>
       </fill>
       <border diagonalUp="0" diagonalDown="0">
@@ -2772,6 +2772,212 @@
         </bottom>
         <vertical/>
         <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -3579,7 +3785,7 @@
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
       <border diagonalUp="0" diagonalDown="0">
@@ -3593,212 +3799,6 @@
         </bottom>
         <vertical/>
         <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -4045,42 +4045,42 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{690E7B34-75E3-43BA-8CDD-44A4EFCCEFD5}" name="Table2" displayName="Table2" ref="A1:AB132" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{690E7B34-75E3-43BA-8CDD-44A4EFCCEFD5}" name="Table2" displayName="Table2" ref="A1:AB132" totalsRowShown="0" headerRowDxfId="46" dataDxfId="45">
   <autoFilter ref="A1:AB132" xr:uid="{690E7B34-75E3-43BA-8CDD-44A4EFCCEFD5}"/>
   <tableColumns count="28">
-    <tableColumn id="9" xr3:uid="{1DBBD25D-72F9-4A81-9CFA-500505E3628D}" name="ID" dataDxfId="38"/>
-    <tableColumn id="14" xr3:uid="{6844A52F-C967-44C0-BF5C-160C47AB6E64}" name="PRO_ID" dataDxfId="37"/>
-    <tableColumn id="12" xr3:uid="{4EDF1E73-4744-474F-8DFE-7F72FB05613C}" name="EPD_ID" dataDxfId="36"/>
-    <tableColumn id="1" xr3:uid="{1CF2E22E-1020-4F35-B31F-6350A15A5DE8}" name="SOURCE" dataDxfId="35"/>
-    <tableColumn id="27" xr3:uid="{07F74D5D-9130-4120-B02C-A11234427F46}" name="KBOB ID-Nr." dataDxfId="34"/>
-    <tableColumn id="11" xr3:uid="{81FE7F31-5F54-40F9-B99E-827E048F7DB5}" name="EPD_DATE" dataDxfId="33"/>
-    <tableColumn id="10" xr3:uid="{54D8BA04-0FEF-4C3B-9B14-59E8F982CD3F}" name="VALID_TO" dataDxfId="32"/>
-    <tableColumn id="22" xr3:uid="{3D6FC370-B8A8-40C3-9FC8-791B178DDFDF}" name="COUNTRY" dataDxfId="31"/>
-    <tableColumn id="4" xr3:uid="{25C7280F-4E3E-4E39-BDBB-DC06DF090C5B}" name="PRODUCT_NAME" dataDxfId="30"/>
-    <tableColumn id="26" xr3:uid="{1053A7DD-B11F-4E75-92EC-BC0F866E90B4}" name="OEKOBAUDAT_ID" dataDxfId="29"/>
-    <tableColumn id="25" xr3:uid="{295F99F8-E318-45C9-833E-F0B45A26471A}" name="MATERIAL_GROUP" dataDxfId="28"/>
-    <tableColumn id="2" xr3:uid="{1326FCEF-D1EE-4F3A-BB8B-77CB4EC72B0C}" name="MATERIAL" dataDxfId="27"/>
-    <tableColumn id="5" xr3:uid="{9B2A7F84-D968-4A00-B61F-23BB0661E7A3}" name="CEMENT" dataDxfId="26"/>
-    <tableColumn id="6" xr3:uid="{2F6E5831-6238-4360-9CFD-ED23A193E761}" name="MECH_PROP" dataDxfId="25"/>
-    <tableColumn id="13" xr3:uid="{50DAB01C-8AF5-4E0C-9904-54F70B81BC55}" name="DENSITY" dataDxfId="24"/>
-    <tableColumn id="18" xr3:uid="{F799A4D4-9543-475F-989E-CFBA47249558}" name="EXPOSITIONSKLASSE" dataDxfId="23"/>
-    <tableColumn id="17" xr3:uid="{ECCBC067-991C-4C60-942D-806BCD77B990}" name="GROESSTKORN" dataDxfId="22"/>
-    <tableColumn id="16" xr3:uid="{05157B85-D5FB-4844-9B53-D8AB09BCE0D9}" name="CHLORIDGEHALT" dataDxfId="21"/>
-    <tableColumn id="15" xr3:uid="{9F53CF50-7148-405A-9295-1F0C3C45645A}" name="KONSISTENZKLASSE" dataDxfId="20"/>
-    <tableColumn id="7" xr3:uid="{E23232F6-E86E-4AD2-8257-F30C0D1F7368}" name="Total_GWP" dataDxfId="19"/>
-    <tableColumn id="20" xr3:uid="{0A9001B4-3AB4-4C58-B125-0B2AA4DB2681}" name="A1toA3_GWP" dataDxfId="18">
+    <tableColumn id="9" xr3:uid="{1DBBD25D-72F9-4A81-9CFA-500505E3628D}" name="ID" dataDxfId="44"/>
+    <tableColumn id="14" xr3:uid="{6844A52F-C967-44C0-BF5C-160C47AB6E64}" name="PRO_ID" dataDxfId="43"/>
+    <tableColumn id="12" xr3:uid="{4EDF1E73-4744-474F-8DFE-7F72FB05613C}" name="EPD_ID" dataDxfId="42"/>
+    <tableColumn id="1" xr3:uid="{1CF2E22E-1020-4F35-B31F-6350A15A5DE8}" name="SOURCE" dataDxfId="41"/>
+    <tableColumn id="27" xr3:uid="{07F74D5D-9130-4120-B02C-A11234427F46}" name="KBOB ID-Nr." dataDxfId="40"/>
+    <tableColumn id="11" xr3:uid="{81FE7F31-5F54-40F9-B99E-827E048F7DB5}" name="EPD_DATE" dataDxfId="39"/>
+    <tableColumn id="10" xr3:uid="{54D8BA04-0FEF-4C3B-9B14-59E8F982CD3F}" name="VALID_TO" dataDxfId="38"/>
+    <tableColumn id="22" xr3:uid="{3D6FC370-B8A8-40C3-9FC8-791B178DDFDF}" name="COUNTRY" dataDxfId="37"/>
+    <tableColumn id="4" xr3:uid="{25C7280F-4E3E-4E39-BDBB-DC06DF090C5B}" name="PRODUCT_NAME" dataDxfId="36"/>
+    <tableColumn id="26" xr3:uid="{1053A7DD-B11F-4E75-92EC-BC0F866E90B4}" name="OEKOBAUDAT_ID" dataDxfId="35"/>
+    <tableColumn id="25" xr3:uid="{295F99F8-E318-45C9-833E-F0B45A26471A}" name="MATERIAL_GROUP" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{1326FCEF-D1EE-4F3A-BB8B-77CB4EC72B0C}" name="MATERIAL" dataDxfId="33"/>
+    <tableColumn id="5" xr3:uid="{9B2A7F84-D968-4A00-B61F-23BB0661E7A3}" name="CEMENT" dataDxfId="32"/>
+    <tableColumn id="6" xr3:uid="{2F6E5831-6238-4360-9CFD-ED23A193E761}" name="MECH_PROP" dataDxfId="31"/>
+    <tableColumn id="13" xr3:uid="{50DAB01C-8AF5-4E0C-9904-54F70B81BC55}" name="DENSITY" dataDxfId="30"/>
+    <tableColumn id="18" xr3:uid="{F799A4D4-9543-475F-989E-CFBA47249558}" name="EXPOSITIONSKLASSE" dataDxfId="29"/>
+    <tableColumn id="17" xr3:uid="{ECCBC067-991C-4C60-942D-806BCD77B990}" name="GROESSTKORN" dataDxfId="28"/>
+    <tableColumn id="16" xr3:uid="{05157B85-D5FB-4844-9B53-D8AB09BCE0D9}" name="CHLORIDGEHALT" dataDxfId="27"/>
+    <tableColumn id="15" xr3:uid="{9F53CF50-7148-405A-9295-1F0C3C45645A}" name="KONSISTENZKLASSE" dataDxfId="26"/>
+    <tableColumn id="7" xr3:uid="{E23232F6-E86E-4AD2-8257-F30C0D1F7368}" name="Total_GWP" dataDxfId="25"/>
+    <tableColumn id="20" xr3:uid="{0A9001B4-3AB4-4C58-B125-0B2AA4DB2681}" name="A1toA3_GWP" dataDxfId="24">
       <calculatedColumnFormula>119+10.9+238</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="21" xr3:uid="{2799394A-C481-45CE-B194-AAABAB0AED38}" name="C1toC4_GWP" dataDxfId="17">
+    <tableColumn id="21" xr3:uid="{2799394A-C481-45CE-B194-AAABAB0AED38}" name="C1toC4_GWP" dataDxfId="23">
       <calculatedColumnFormula>51.1+26+2.64+12.6</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="19" xr3:uid="{70561D70-9D02-4E93-A395-229DA8696DDA}" name="ValidEPD" dataDxfId="16">
+    <tableColumn id="19" xr3:uid="{70561D70-9D02-4E93-A395-229DA8696DDA}" name="ValidEPD" dataDxfId="22">
       <calculatedColumnFormula>IF(OR($D2="Ecoinvent",$D2="Betonsortenrechner",$D2="KBOB",$T2&lt;=0),0,1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="29" xr3:uid="{92D55BC7-F55B-406A-B127-69EC2F0A8B77}" name="noch gültig" dataDxfId="15">
+    <tableColumn id="29" xr3:uid="{92D55BC7-F55B-406A-B127-69EC2F0A8B77}" name="noch gültig" dataDxfId="21">
       <calculatedColumnFormula>IF(Table2[[#This Row],[VALID_TO]]&gt;=TODAY(), 1, 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{DB90AC0A-8933-4040-BADE-E6EE11AC8BD7}" name="Statistik" dataDxfId="14">
+    <tableColumn id="3" xr3:uid="{DB90AC0A-8933-4040-BADE-E6EE11AC8BD7}" name="Statistik" dataDxfId="20">
       <calculatedColumnFormula array="1">IF($W2&lt;&gt;0,
 IF(AND(
                          T2&gt;=_xlfn.PERCENTILE.INC(_xlfn._xlws.FILTER($T$2:$T$148, ($L$2:$L$148=L2)*($W$2:$W$148=1)),0.1),
@@ -4088,41 +4088,41 @@
                ),1,0),
 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{BBA6C134-63F9-4711-8B25-086098EC2CB0}" name="Cost" dataDxfId="13"/>
-    <tableColumn id="24" xr3:uid="{5321A0E1-043C-4E95-A6DA-41830364B2BC}" name="Anmerkung" dataDxfId="12"/>
-    <tableColumn id="23" xr3:uid="{61456234-34E8-4222-B2D6-9DDA8E83B081}" name="Spalte 1" dataDxfId="11"/>
+    <tableColumn id="8" xr3:uid="{BBA6C134-63F9-4711-8B25-086098EC2CB0}" name="Cost" dataDxfId="19"/>
+    <tableColumn id="24" xr3:uid="{5321A0E1-043C-4E95-A6DA-41830364B2BC}" name="Anmerkung" dataDxfId="18"/>
+    <tableColumn id="23" xr3:uid="{61456234-34E8-4222-B2D6-9DDA8E83B081}" name="Spalte 1" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{188FAA96-3B75-4826-B66B-A81D5BCFC670}" name="Tabelle4" displayName="Tabelle4" ref="A1:J8" totalsRowShown="0" headerRowDxfId="55" dataDxfId="53" headerRowBorderDxfId="54" tableBorderDxfId="52" totalsRowBorderDxfId="51">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{188FAA96-3B75-4826-B66B-A81D5BCFC670}" name="Tabelle4" displayName="Tabelle4" ref="A1:J8" totalsRowShown="0" headerRowDxfId="16" dataDxfId="14" headerRowBorderDxfId="15" tableBorderDxfId="13" totalsRowBorderDxfId="12">
   <autoFilter ref="A1:J8" xr:uid="{188FAA96-3B75-4826-B66B-A81D5BCFC670}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{AF3C694B-2C8A-40EE-B8BB-2EC9EB81A87A}" name="mat_ID" dataDxfId="50"/>
-    <tableColumn id="2" xr3:uid="{B447FBC2-C455-4332-8F47-150B112A57E0}" name="name" dataDxfId="49"/>
-    <tableColumn id="3" xr3:uid="{BAFC6B47-7268-46CC-A881-892C9A1F4334}" name="strength_comp" dataDxfId="48"/>
-    <tableColumn id="4" xr3:uid="{6FC4C8EB-7581-4E67-81CE-C724161F0838}" name="strength_tens" dataDxfId="47"/>
-    <tableColumn id="5" xr3:uid="{A875970E-61A9-43B5-9361-7616A74C3147}" name="strength_bend" dataDxfId="46"/>
-    <tableColumn id="6" xr3:uid="{EF5B3A69-DD70-420A-88FF-4FE8772A2E14}" name="strength_shea" dataDxfId="45"/>
-    <tableColumn id="7" xr3:uid="{ED461A80-736C-42BD-81BC-C5C0C80FF34C}" name="E_modulus" dataDxfId="44"/>
-    <tableColumn id="8" xr3:uid="{68E47481-7028-4427-B126-2A046FC46737}" name="density_load" dataDxfId="43"/>
-    <tableColumn id="9" xr3:uid="{7AB34570-2BD4-417F-B141-70612577C7D6}" name="burn_rate" dataDxfId="42"/>
-    <tableColumn id="10" xr3:uid="{69298654-E280-9D4B-9717-7904FADC15B5}" name="phi" dataDxfId="41"/>
+    <tableColumn id="1" xr3:uid="{AF3C694B-2C8A-40EE-B8BB-2EC9EB81A87A}" name="mat_ID" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{B447FBC2-C455-4332-8F47-150B112A57E0}" name="name" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{BAFC6B47-7268-46CC-A881-892C9A1F4334}" name="strength_comp" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{6FC4C8EB-7581-4E67-81CE-C724161F0838}" name="strength_tens" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{A875970E-61A9-43B5-9361-7616A74C3147}" name="strength_bend" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{EF5B3A69-DD70-420A-88FF-4FE8772A2E14}" name="strength_shea" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{ED461A80-736C-42BD-81BC-C5C0C80FF34C}" name="E_modulus" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{68E47481-7028-4427-B126-2A046FC46737}" name="density_load" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{7AB34570-2BD4-417F-B141-70612577C7D6}" name="burn_rate" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{69298654-E280-9D4B-9717-7904FADC15B5}" name="phi" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1CD264FD-E2C0-E94F-B387-736226CC982D}" name="Tabelle42" displayName="Tabelle42" ref="A1:D6" totalsRowShown="0" headerRowDxfId="10" dataDxfId="8" headerRowBorderDxfId="9" tableBorderDxfId="7" totalsRowBorderDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1CD264FD-E2C0-E94F-B387-736226CC982D}" name="Tabelle42" displayName="Tabelle42" ref="A1:D6" totalsRowShown="0" headerRowDxfId="55" dataDxfId="53" headerRowBorderDxfId="54" tableBorderDxfId="52" totalsRowBorderDxfId="51">
   <autoFilter ref="A1:D6" xr:uid="{1CD264FD-E2C0-E94F-B387-736226CC982D}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{6590463D-C242-4C4D-AA1F-6FA1F0D35E6F}" name="mat_ID" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{603BAED4-55F2-D040-9D73-1611C1564A84}" name="name" dataDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{D6CC67C0-1ACA-D446-A6F3-00BCC3AC8DAC}" name="d" dataDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{3D62C7FF-3D7F-B245-A874-3A95DF0C49D2}" name="K_ser" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{6590463D-C242-4C4D-AA1F-6FA1F0D35E6F}" name="mat_ID" dataDxfId="50"/>
+    <tableColumn id="2" xr3:uid="{603BAED4-55F2-D040-9D73-1611C1564A84}" name="name" dataDxfId="49"/>
+    <tableColumn id="3" xr3:uid="{D6CC67C0-1ACA-D446-A6F3-00BCC3AC8DAC}" name="d" dataDxfId="48"/>
+    <tableColumn id="4" xr3:uid="{3D62C7FF-3D7F-B245-A874-3A95DF0C49D2}" name="K_ser" dataDxfId="47"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -16191,6 +16191,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBA60A30-8D92-49EC-964A-A8F2973B4787}">
   <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="33.33203125" customWidth="1"/>
+    <col min="3" max="3" width="19.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">

</xml_diff>

<commit_message>
Added TCC concrete slab fire check
</commit_message>
<xml_diff>
--- a/Database/260126_Datenbankdefinition.xlsx
+++ b/Database/260126_Datenbankdefinition.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jonathanbieg/Documents/Master Thesis/1_Code/Python Repository/SDSD_Bieg/Database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{451D9134-3CDB-794D-A94C-48E9C3B75C34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31B64A7D-A041-C441-A85B-212128E48FB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="600" yWindow="840" windowWidth="25180" windowHeight="16700" activeTab="3" xr2:uid="{58B6788A-438B-478E-898A-D53025B55ED1}"/>
+    <workbookView xWindow="600" yWindow="840" windowWidth="25180" windowHeight="16700" activeTab="2" xr2:uid="{58B6788A-438B-478E-898A-D53025B55ED1}"/>
   </bookViews>
   <sheets>
     <sheet name="products" sheetId="1" r:id="rId1"/>
@@ -16194,6 +16194,8 @@
   <cols>
     <col min="2" max="2" width="33.33203125" customWidth="1"/>
     <col min="3" max="3" width="19.6640625" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
     <col min="7" max="7" width="30" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
class PostTensionedConcrete: Added mr and EIeff
</commit_message>
<xml_diff>
--- a/Database/260126_Datenbankdefinition.xlsx
+++ b/Database/260126_Datenbankdefinition.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jonathanbieg/Documents/Master Thesis/1_Code/Python Repository/SDSD_Bieg/Database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A0D5814-88E2-FF43-84D8-35F857464BF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D943D0A5-A188-A14A-B5BD-62BE563A0ABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17160" xr2:uid="{58B6788A-438B-478E-898A-D53025B55ED1}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17160" activeTab="1" xr2:uid="{58B6788A-438B-478E-898A-D53025B55ED1}"/>
   </bookViews>
   <sheets>
     <sheet name="products" sheetId="1" r:id="rId1"/>
@@ -3012,6 +3012,422 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
@@ -3649,422 +4065,6 @@
       </font>
       <alignment vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4"/>
-          <bgColor theme="4"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -4135,42 +4135,42 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{690E7B34-75E3-43BA-8CDD-44A4EFCCEFD5}" name="Table2" displayName="Table2" ref="A1:AC132" totalsRowShown="0" headerRowDxfId="43" dataDxfId="42">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{690E7B34-75E3-43BA-8CDD-44A4EFCCEFD5}" name="Table2" displayName="Table2" ref="A1:AC132" totalsRowShown="0" headerRowDxfId="58" dataDxfId="57">
   <autoFilter ref="A1:AC132" xr:uid="{690E7B34-75E3-43BA-8CDD-44A4EFCCEFD5}"/>
   <tableColumns count="29">
-    <tableColumn id="9" xr3:uid="{1DBBD25D-72F9-4A81-9CFA-500505E3628D}" name="ID" dataDxfId="41"/>
-    <tableColumn id="14" xr3:uid="{6844A52F-C967-44C0-BF5C-160C47AB6E64}" name="PRO_ID" dataDxfId="40"/>
-    <tableColumn id="12" xr3:uid="{4EDF1E73-4744-474F-8DFE-7F72FB05613C}" name="EPD_ID" dataDxfId="39"/>
-    <tableColumn id="1" xr3:uid="{1CF2E22E-1020-4F35-B31F-6350A15A5DE8}" name="SOURCE" dataDxfId="38"/>
-    <tableColumn id="27" xr3:uid="{07F74D5D-9130-4120-B02C-A11234427F46}" name="KBOB ID-Nr." dataDxfId="37"/>
-    <tableColumn id="11" xr3:uid="{81FE7F31-5F54-40F9-B99E-827E048F7DB5}" name="EPD_DATE" dataDxfId="36"/>
-    <tableColumn id="10" xr3:uid="{54D8BA04-0FEF-4C3B-9B14-59E8F982CD3F}" name="VALID_TO" dataDxfId="35"/>
-    <tableColumn id="22" xr3:uid="{3D6FC370-B8A8-40C3-9FC8-791B178DDFDF}" name="COUNTRY" dataDxfId="34"/>
-    <tableColumn id="4" xr3:uid="{25C7280F-4E3E-4E39-BDBB-DC06DF090C5B}" name="PRODUCT_NAME" dataDxfId="33"/>
-    <tableColumn id="26" xr3:uid="{1053A7DD-B11F-4E75-92EC-BC0F866E90B4}" name="OEKOBAUDAT_ID" dataDxfId="32"/>
-    <tableColumn id="25" xr3:uid="{295F99F8-E318-45C9-833E-F0B45A26471A}" name="MATERIAL_GROUP" dataDxfId="31"/>
-    <tableColumn id="2" xr3:uid="{1326FCEF-D1EE-4F3A-BB8B-77CB4EC72B0C}" name="MATERIAL" dataDxfId="30"/>
-    <tableColumn id="5" xr3:uid="{9B2A7F84-D968-4A00-B61F-23BB0661E7A3}" name="CEMENT" dataDxfId="29"/>
-    <tableColumn id="6" xr3:uid="{2F6E5831-6238-4360-9CFD-ED23A193E761}" name="MECH_PROP" dataDxfId="28"/>
-    <tableColumn id="13" xr3:uid="{50DAB01C-8AF5-4E0C-9904-54F70B81BC55}" name="DENSITY" dataDxfId="27"/>
-    <tableColumn id="18" xr3:uid="{F799A4D4-9543-475F-989E-CFBA47249558}" name="EXPOSITIONSKLASSE" dataDxfId="26"/>
-    <tableColumn id="17" xr3:uid="{ECCBC067-991C-4C60-942D-806BCD77B990}" name="GROESSTKORN" dataDxfId="25"/>
-    <tableColumn id="16" xr3:uid="{05157B85-D5FB-4844-9B53-D8AB09BCE0D9}" name="CHLORIDGEHALT" dataDxfId="24"/>
-    <tableColumn id="15" xr3:uid="{9F53CF50-7148-405A-9295-1F0C3C45645A}" name="KONSISTENZKLASSE" dataDxfId="23"/>
-    <tableColumn id="7" xr3:uid="{E23232F6-E86E-4AD2-8257-F30C0D1F7368}" name="Total_GWP" dataDxfId="22"/>
-    <tableColumn id="20" xr3:uid="{0A9001B4-3AB4-4C58-B125-0B2AA4DB2681}" name="A1toA3_GWP" dataDxfId="21">
+    <tableColumn id="9" xr3:uid="{1DBBD25D-72F9-4A81-9CFA-500505E3628D}" name="ID" dataDxfId="56"/>
+    <tableColumn id="14" xr3:uid="{6844A52F-C967-44C0-BF5C-160C47AB6E64}" name="PRO_ID" dataDxfId="55"/>
+    <tableColumn id="12" xr3:uid="{4EDF1E73-4744-474F-8DFE-7F72FB05613C}" name="EPD_ID" dataDxfId="54"/>
+    <tableColumn id="1" xr3:uid="{1CF2E22E-1020-4F35-B31F-6350A15A5DE8}" name="SOURCE" dataDxfId="53"/>
+    <tableColumn id="27" xr3:uid="{07F74D5D-9130-4120-B02C-A11234427F46}" name="KBOB ID-Nr." dataDxfId="52"/>
+    <tableColumn id="11" xr3:uid="{81FE7F31-5F54-40F9-B99E-827E048F7DB5}" name="EPD_DATE" dataDxfId="51"/>
+    <tableColumn id="10" xr3:uid="{54D8BA04-0FEF-4C3B-9B14-59E8F982CD3F}" name="VALID_TO" dataDxfId="50"/>
+    <tableColumn id="22" xr3:uid="{3D6FC370-B8A8-40C3-9FC8-791B178DDFDF}" name="COUNTRY" dataDxfId="49"/>
+    <tableColumn id="4" xr3:uid="{25C7280F-4E3E-4E39-BDBB-DC06DF090C5B}" name="PRODUCT_NAME" dataDxfId="48"/>
+    <tableColumn id="26" xr3:uid="{1053A7DD-B11F-4E75-92EC-BC0F866E90B4}" name="OEKOBAUDAT_ID" dataDxfId="47"/>
+    <tableColumn id="25" xr3:uid="{295F99F8-E318-45C9-833E-F0B45A26471A}" name="MATERIAL_GROUP" dataDxfId="46"/>
+    <tableColumn id="2" xr3:uid="{1326FCEF-D1EE-4F3A-BB8B-77CB4EC72B0C}" name="MATERIAL" dataDxfId="45"/>
+    <tableColumn id="5" xr3:uid="{9B2A7F84-D968-4A00-B61F-23BB0661E7A3}" name="CEMENT" dataDxfId="44"/>
+    <tableColumn id="6" xr3:uid="{2F6E5831-6238-4360-9CFD-ED23A193E761}" name="MECH_PROP" dataDxfId="43"/>
+    <tableColumn id="13" xr3:uid="{50DAB01C-8AF5-4E0C-9904-54F70B81BC55}" name="DENSITY" dataDxfId="42"/>
+    <tableColumn id="18" xr3:uid="{F799A4D4-9543-475F-989E-CFBA47249558}" name="EXPOSITIONSKLASSE" dataDxfId="41"/>
+    <tableColumn id="17" xr3:uid="{ECCBC067-991C-4C60-942D-806BCD77B990}" name="GROESSTKORN" dataDxfId="40"/>
+    <tableColumn id="16" xr3:uid="{05157B85-D5FB-4844-9B53-D8AB09BCE0D9}" name="CHLORIDGEHALT" dataDxfId="39"/>
+    <tableColumn id="15" xr3:uid="{9F53CF50-7148-405A-9295-1F0C3C45645A}" name="KONSISTENZKLASSE" dataDxfId="38"/>
+    <tableColumn id="7" xr3:uid="{E23232F6-E86E-4AD2-8257-F30C0D1F7368}" name="Total_GWP" dataDxfId="37"/>
+    <tableColumn id="20" xr3:uid="{0A9001B4-3AB4-4C58-B125-0B2AA4DB2681}" name="A1toA3_GWP" dataDxfId="36">
       <calculatedColumnFormula>119+10.9+238</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="21" xr3:uid="{2799394A-C481-45CE-B194-AAABAB0AED38}" name="C1toC4_GWP" dataDxfId="20">
+    <tableColumn id="21" xr3:uid="{2799394A-C481-45CE-B194-AAABAB0AED38}" name="C1toC4_GWP" dataDxfId="35">
       <calculatedColumnFormula>51.1+26+2.64+12.6</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="19" xr3:uid="{70561D70-9D02-4E93-A395-229DA8696DDA}" name="ValidEPD" dataDxfId="19">
+    <tableColumn id="19" xr3:uid="{70561D70-9D02-4E93-A395-229DA8696DDA}" name="ValidEPD" dataDxfId="34">
       <calculatedColumnFormula>IF(OR($D2="Ecoinvent",$D2="Betonsortenrechner",$D2="KBOB",$T2&lt;=0),0,1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="29" xr3:uid="{92D55BC7-F55B-406A-B127-69EC2F0A8B77}" name="noch gültig" dataDxfId="18">
+    <tableColumn id="29" xr3:uid="{92D55BC7-F55B-406A-B127-69EC2F0A8B77}" name="noch gültig" dataDxfId="33">
       <calculatedColumnFormula>IF(Table2[[#This Row],[VALID_TO]]&gt;=TODAY(), 1, 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{DB90AC0A-8933-4040-BADE-E6EE11AC8BD7}" name="Statistik" dataDxfId="17">
+    <tableColumn id="3" xr3:uid="{DB90AC0A-8933-4040-BADE-E6EE11AC8BD7}" name="Statistik" dataDxfId="32">
       <calculatedColumnFormula array="1">IF($W2&lt;&gt;0,
 IF(AND(
                          T2&gt;=_xlfn.PERCENTILE.INC(_xlfn._xlws.FILTER($T$2:$T$148, ($L$2:$L$148=L2)*($W$2:$W$148=1)),0.1),
@@ -4178,29 +4178,29 @@
                ),1,0),
 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{BBA6C134-63F9-4711-8B25-086098EC2CB0}" name="Cost" dataDxfId="16"/>
-    <tableColumn id="24" xr3:uid="{5321A0E1-043C-4E95-A6DA-41830364B2BC}" name="Anmerkung" dataDxfId="15"/>
-    <tableColumn id="23" xr3:uid="{61456234-34E8-4222-B2D6-9DDA8E83B081}" name="Spalte 1" dataDxfId="14"/>
-    <tableColumn id="28" xr3:uid="{D1FC9AF8-A0AE-CE49-8F27-4BB569415BF3}" name="T_construction" dataDxfId="13"/>
+    <tableColumn id="8" xr3:uid="{BBA6C134-63F9-4711-8B25-086098EC2CB0}" name="Cost" dataDxfId="31"/>
+    <tableColumn id="24" xr3:uid="{5321A0E1-043C-4E95-A6DA-41830364B2BC}" name="Anmerkung" dataDxfId="30"/>
+    <tableColumn id="23" xr3:uid="{61456234-34E8-4222-B2D6-9DDA8E83B081}" name="Spalte 1" dataDxfId="29"/>
+    <tableColumn id="28" xr3:uid="{D1FC9AF8-A0AE-CE49-8F27-4BB569415BF3}" name="T_construction" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{188FAA96-3B75-4826-B66B-A81D5BCFC670}" name="Tabelle4" displayName="Tabelle4" ref="A1:J9" totalsRowShown="0" headerRowDxfId="58" dataDxfId="56" headerRowBorderDxfId="57" tableBorderDxfId="55" totalsRowBorderDxfId="54">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{188FAA96-3B75-4826-B66B-A81D5BCFC670}" name="Tabelle4" displayName="Tabelle4" ref="A1:J9" totalsRowShown="0" headerRowDxfId="27" dataDxfId="25" headerRowBorderDxfId="26" tableBorderDxfId="24" totalsRowBorderDxfId="23">
   <autoFilter ref="A1:J9" xr:uid="{188FAA96-3B75-4826-B66B-A81D5BCFC670}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{AF3C694B-2C8A-40EE-B8BB-2EC9EB81A87A}" name="mat_ID" dataDxfId="53"/>
-    <tableColumn id="2" xr3:uid="{B447FBC2-C455-4332-8F47-150B112A57E0}" name="name" dataDxfId="52"/>
-    <tableColumn id="3" xr3:uid="{BAFC6B47-7268-46CC-A881-892C9A1F4334}" name="strength_comp" dataDxfId="51"/>
-    <tableColumn id="4" xr3:uid="{6FC4C8EB-7581-4E67-81CE-C724161F0838}" name="strength_tens" dataDxfId="50"/>
-    <tableColumn id="5" xr3:uid="{A875970E-61A9-43B5-9361-7616A74C3147}" name="strength_bend" dataDxfId="49"/>
-    <tableColumn id="6" xr3:uid="{EF5B3A69-DD70-420A-88FF-4FE8772A2E14}" name="strength_shea" dataDxfId="48"/>
-    <tableColumn id="7" xr3:uid="{ED461A80-736C-42BD-81BC-C5C0C80FF34C}" name="E_modulus" dataDxfId="47"/>
-    <tableColumn id="8" xr3:uid="{68E47481-7028-4427-B126-2A046FC46737}" name="density_load" dataDxfId="46"/>
-    <tableColumn id="9" xr3:uid="{7AB34570-2BD4-417F-B141-70612577C7D6}" name="burn_rate" dataDxfId="45"/>
-    <tableColumn id="10" xr3:uid="{69298654-E280-9D4B-9717-7904FADC15B5}" name="phi" dataDxfId="44"/>
+    <tableColumn id="1" xr3:uid="{AF3C694B-2C8A-40EE-B8BB-2EC9EB81A87A}" name="mat_ID" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{B447FBC2-C455-4332-8F47-150B112A57E0}" name="name" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{BAFC6B47-7268-46CC-A881-892C9A1F4334}" name="strength_comp" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{6FC4C8EB-7581-4E67-81CE-C724161F0838}" name="strength_tens" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{A875970E-61A9-43B5-9361-7616A74C3147}" name="strength_bend" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{EF5B3A69-DD70-420A-88FF-4FE8772A2E14}" name="strength_shea" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{ED461A80-736C-42BD-81BC-C5C0C80FF34C}" name="E_modulus" dataDxfId="16"/>
+    <tableColumn id="8" xr3:uid="{68E47481-7028-4427-B126-2A046FC46737}" name="density_load" dataDxfId="15"/>
+    <tableColumn id="9" xr3:uid="{7AB34570-2BD4-417F-B141-70612577C7D6}" name="burn_rate" dataDxfId="14"/>
+    <tableColumn id="10" xr3:uid="{69298654-E280-9D4B-9717-7904FADC15B5}" name="phi" dataDxfId="13"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -17048,7 +17048,7 @@
       </c>
       <c r="C9" s="62"/>
       <c r="D9" s="62">
-        <v>1600000000</v>
+        <v>1860000000</v>
       </c>
       <c r="E9" s="62"/>
       <c r="F9" s="62"/>

</xml_diff>

<commit_message>
Added punching handling and pt Member2D handling
</commit_message>
<xml_diff>
--- a/Database/260126_Datenbankdefinition.xlsx
+++ b/Database/260126_Datenbankdefinition.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -3012,422 +3012,6 @@
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4"/>
-          <bgColor theme="4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <strike val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
@@ -4065,6 +3649,422 @@
       </font>
       <alignment vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -4135,42 +4135,42 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{690E7B34-75E3-43BA-8CDD-44A4EFCCEFD5}" name="Table2" displayName="Table2" ref="A1:AC132" totalsRowShown="0" headerRowDxfId="58" dataDxfId="57">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{690E7B34-75E3-43BA-8CDD-44A4EFCCEFD5}" name="Table2" displayName="Table2" ref="A1:AC132" totalsRowShown="0" headerRowDxfId="43" dataDxfId="42">
   <autoFilter ref="A1:AC132" xr:uid="{690E7B34-75E3-43BA-8CDD-44A4EFCCEFD5}"/>
   <tableColumns count="29">
-    <tableColumn id="9" xr3:uid="{1DBBD25D-72F9-4A81-9CFA-500505E3628D}" name="ID" dataDxfId="56"/>
-    <tableColumn id="14" xr3:uid="{6844A52F-C967-44C0-BF5C-160C47AB6E64}" name="PRO_ID" dataDxfId="55"/>
-    <tableColumn id="12" xr3:uid="{4EDF1E73-4744-474F-8DFE-7F72FB05613C}" name="EPD_ID" dataDxfId="54"/>
-    <tableColumn id="1" xr3:uid="{1CF2E22E-1020-4F35-B31F-6350A15A5DE8}" name="SOURCE" dataDxfId="53"/>
-    <tableColumn id="27" xr3:uid="{07F74D5D-9130-4120-B02C-A11234427F46}" name="KBOB ID-Nr." dataDxfId="52"/>
-    <tableColumn id="11" xr3:uid="{81FE7F31-5F54-40F9-B99E-827E048F7DB5}" name="EPD_DATE" dataDxfId="51"/>
-    <tableColumn id="10" xr3:uid="{54D8BA04-0FEF-4C3B-9B14-59E8F982CD3F}" name="VALID_TO" dataDxfId="50"/>
-    <tableColumn id="22" xr3:uid="{3D6FC370-B8A8-40C3-9FC8-791B178DDFDF}" name="COUNTRY" dataDxfId="49"/>
-    <tableColumn id="4" xr3:uid="{25C7280F-4E3E-4E39-BDBB-DC06DF090C5B}" name="PRODUCT_NAME" dataDxfId="48"/>
-    <tableColumn id="26" xr3:uid="{1053A7DD-B11F-4E75-92EC-BC0F866E90B4}" name="OEKOBAUDAT_ID" dataDxfId="47"/>
-    <tableColumn id="25" xr3:uid="{295F99F8-E318-45C9-833E-F0B45A26471A}" name="MATERIAL_GROUP" dataDxfId="46"/>
-    <tableColumn id="2" xr3:uid="{1326FCEF-D1EE-4F3A-BB8B-77CB4EC72B0C}" name="MATERIAL" dataDxfId="45"/>
-    <tableColumn id="5" xr3:uid="{9B2A7F84-D968-4A00-B61F-23BB0661E7A3}" name="CEMENT" dataDxfId="44"/>
-    <tableColumn id="6" xr3:uid="{2F6E5831-6238-4360-9CFD-ED23A193E761}" name="MECH_PROP" dataDxfId="43"/>
-    <tableColumn id="13" xr3:uid="{50DAB01C-8AF5-4E0C-9904-54F70B81BC55}" name="DENSITY" dataDxfId="42"/>
-    <tableColumn id="18" xr3:uid="{F799A4D4-9543-475F-989E-CFBA47249558}" name="EXPOSITIONSKLASSE" dataDxfId="41"/>
-    <tableColumn id="17" xr3:uid="{ECCBC067-991C-4C60-942D-806BCD77B990}" name="GROESSTKORN" dataDxfId="40"/>
-    <tableColumn id="16" xr3:uid="{05157B85-D5FB-4844-9B53-D8AB09BCE0D9}" name="CHLORIDGEHALT" dataDxfId="39"/>
-    <tableColumn id="15" xr3:uid="{9F53CF50-7148-405A-9295-1F0C3C45645A}" name="KONSISTENZKLASSE" dataDxfId="38"/>
-    <tableColumn id="7" xr3:uid="{E23232F6-E86E-4AD2-8257-F30C0D1F7368}" name="Total_GWP" dataDxfId="37"/>
-    <tableColumn id="20" xr3:uid="{0A9001B4-3AB4-4C58-B125-0B2AA4DB2681}" name="A1toA3_GWP" dataDxfId="36">
+    <tableColumn id="9" xr3:uid="{1DBBD25D-72F9-4A81-9CFA-500505E3628D}" name="ID" dataDxfId="41"/>
+    <tableColumn id="14" xr3:uid="{6844A52F-C967-44C0-BF5C-160C47AB6E64}" name="PRO_ID" dataDxfId="40"/>
+    <tableColumn id="12" xr3:uid="{4EDF1E73-4744-474F-8DFE-7F72FB05613C}" name="EPD_ID" dataDxfId="39"/>
+    <tableColumn id="1" xr3:uid="{1CF2E22E-1020-4F35-B31F-6350A15A5DE8}" name="SOURCE" dataDxfId="38"/>
+    <tableColumn id="27" xr3:uid="{07F74D5D-9130-4120-B02C-A11234427F46}" name="KBOB ID-Nr." dataDxfId="37"/>
+    <tableColumn id="11" xr3:uid="{81FE7F31-5F54-40F9-B99E-827E048F7DB5}" name="EPD_DATE" dataDxfId="36"/>
+    <tableColumn id="10" xr3:uid="{54D8BA04-0FEF-4C3B-9B14-59E8F982CD3F}" name="VALID_TO" dataDxfId="35"/>
+    <tableColumn id="22" xr3:uid="{3D6FC370-B8A8-40C3-9FC8-791B178DDFDF}" name="COUNTRY" dataDxfId="34"/>
+    <tableColumn id="4" xr3:uid="{25C7280F-4E3E-4E39-BDBB-DC06DF090C5B}" name="PRODUCT_NAME" dataDxfId="33"/>
+    <tableColumn id="26" xr3:uid="{1053A7DD-B11F-4E75-92EC-BC0F866E90B4}" name="OEKOBAUDAT_ID" dataDxfId="32"/>
+    <tableColumn id="25" xr3:uid="{295F99F8-E318-45C9-833E-F0B45A26471A}" name="MATERIAL_GROUP" dataDxfId="31"/>
+    <tableColumn id="2" xr3:uid="{1326FCEF-D1EE-4F3A-BB8B-77CB4EC72B0C}" name="MATERIAL" dataDxfId="30"/>
+    <tableColumn id="5" xr3:uid="{9B2A7F84-D968-4A00-B61F-23BB0661E7A3}" name="CEMENT" dataDxfId="29"/>
+    <tableColumn id="6" xr3:uid="{2F6E5831-6238-4360-9CFD-ED23A193E761}" name="MECH_PROP" dataDxfId="28"/>
+    <tableColumn id="13" xr3:uid="{50DAB01C-8AF5-4E0C-9904-54F70B81BC55}" name="DENSITY" dataDxfId="27"/>
+    <tableColumn id="18" xr3:uid="{F799A4D4-9543-475F-989E-CFBA47249558}" name="EXPOSITIONSKLASSE" dataDxfId="26"/>
+    <tableColumn id="17" xr3:uid="{ECCBC067-991C-4C60-942D-806BCD77B990}" name="GROESSTKORN" dataDxfId="25"/>
+    <tableColumn id="16" xr3:uid="{05157B85-D5FB-4844-9B53-D8AB09BCE0D9}" name="CHLORIDGEHALT" dataDxfId="24"/>
+    <tableColumn id="15" xr3:uid="{9F53CF50-7148-405A-9295-1F0C3C45645A}" name="KONSISTENZKLASSE" dataDxfId="23"/>
+    <tableColumn id="7" xr3:uid="{E23232F6-E86E-4AD2-8257-F30C0D1F7368}" name="Total_GWP" dataDxfId="22"/>
+    <tableColumn id="20" xr3:uid="{0A9001B4-3AB4-4C58-B125-0B2AA4DB2681}" name="A1toA3_GWP" dataDxfId="21">
       <calculatedColumnFormula>119+10.9+238</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="21" xr3:uid="{2799394A-C481-45CE-B194-AAABAB0AED38}" name="C1toC4_GWP" dataDxfId="35">
+    <tableColumn id="21" xr3:uid="{2799394A-C481-45CE-B194-AAABAB0AED38}" name="C1toC4_GWP" dataDxfId="20">
       <calculatedColumnFormula>51.1+26+2.64+12.6</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="19" xr3:uid="{70561D70-9D02-4E93-A395-229DA8696DDA}" name="ValidEPD" dataDxfId="34">
+    <tableColumn id="19" xr3:uid="{70561D70-9D02-4E93-A395-229DA8696DDA}" name="ValidEPD" dataDxfId="19">
       <calculatedColumnFormula>IF(OR($D2="Ecoinvent",$D2="Betonsortenrechner",$D2="KBOB",$T2&lt;=0),0,1)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="29" xr3:uid="{92D55BC7-F55B-406A-B127-69EC2F0A8B77}" name="noch gültig" dataDxfId="33">
+    <tableColumn id="29" xr3:uid="{92D55BC7-F55B-406A-B127-69EC2F0A8B77}" name="noch gültig" dataDxfId="18">
       <calculatedColumnFormula>IF(Table2[[#This Row],[VALID_TO]]&gt;=TODAY(), 1, 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{DB90AC0A-8933-4040-BADE-E6EE11AC8BD7}" name="Statistik" dataDxfId="32">
+    <tableColumn id="3" xr3:uid="{DB90AC0A-8933-4040-BADE-E6EE11AC8BD7}" name="Statistik" dataDxfId="17">
       <calculatedColumnFormula array="1">IF($W2&lt;&gt;0,
 IF(AND(
                          T2&gt;=_xlfn.PERCENTILE.INC(_xlfn._xlws.FILTER($T$2:$T$148, ($L$2:$L$148=L2)*($W$2:$W$148=1)),0.1),
@@ -4178,29 +4178,29 @@
                ),1,0),
 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{BBA6C134-63F9-4711-8B25-086098EC2CB0}" name="Cost" dataDxfId="31"/>
-    <tableColumn id="24" xr3:uid="{5321A0E1-043C-4E95-A6DA-41830364B2BC}" name="Anmerkung" dataDxfId="30"/>
-    <tableColumn id="23" xr3:uid="{61456234-34E8-4222-B2D6-9DDA8E83B081}" name="Spalte 1" dataDxfId="29"/>
-    <tableColumn id="28" xr3:uid="{D1FC9AF8-A0AE-CE49-8F27-4BB569415BF3}" name="T_construction" dataDxfId="28"/>
+    <tableColumn id="8" xr3:uid="{BBA6C134-63F9-4711-8B25-086098EC2CB0}" name="Cost" dataDxfId="16"/>
+    <tableColumn id="24" xr3:uid="{5321A0E1-043C-4E95-A6DA-41830364B2BC}" name="Anmerkung" dataDxfId="15"/>
+    <tableColumn id="23" xr3:uid="{61456234-34E8-4222-B2D6-9DDA8E83B081}" name="Spalte 1" dataDxfId="14"/>
+    <tableColumn id="28" xr3:uid="{D1FC9AF8-A0AE-CE49-8F27-4BB569415BF3}" name="T_construction" dataDxfId="13"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{188FAA96-3B75-4826-B66B-A81D5BCFC670}" name="Tabelle4" displayName="Tabelle4" ref="A1:J9" totalsRowShown="0" headerRowDxfId="27" dataDxfId="25" headerRowBorderDxfId="26" tableBorderDxfId="24" totalsRowBorderDxfId="23">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{188FAA96-3B75-4826-B66B-A81D5BCFC670}" name="Tabelle4" displayName="Tabelle4" ref="A1:J9" totalsRowShown="0" headerRowDxfId="58" dataDxfId="56" headerRowBorderDxfId="57" tableBorderDxfId="55" totalsRowBorderDxfId="54">
   <autoFilter ref="A1:J9" xr:uid="{188FAA96-3B75-4826-B66B-A81D5BCFC670}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{AF3C694B-2C8A-40EE-B8BB-2EC9EB81A87A}" name="mat_ID" dataDxfId="22"/>
-    <tableColumn id="2" xr3:uid="{B447FBC2-C455-4332-8F47-150B112A57E0}" name="name" dataDxfId="21"/>
-    <tableColumn id="3" xr3:uid="{BAFC6B47-7268-46CC-A881-892C9A1F4334}" name="strength_comp" dataDxfId="20"/>
-    <tableColumn id="4" xr3:uid="{6FC4C8EB-7581-4E67-81CE-C724161F0838}" name="strength_tens" dataDxfId="19"/>
-    <tableColumn id="5" xr3:uid="{A875970E-61A9-43B5-9361-7616A74C3147}" name="strength_bend" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{EF5B3A69-DD70-420A-88FF-4FE8772A2E14}" name="strength_shea" dataDxfId="17"/>
-    <tableColumn id="7" xr3:uid="{ED461A80-736C-42BD-81BC-C5C0C80FF34C}" name="E_modulus" dataDxfId="16"/>
-    <tableColumn id="8" xr3:uid="{68E47481-7028-4427-B126-2A046FC46737}" name="density_load" dataDxfId="15"/>
-    <tableColumn id="9" xr3:uid="{7AB34570-2BD4-417F-B141-70612577C7D6}" name="burn_rate" dataDxfId="14"/>
-    <tableColumn id="10" xr3:uid="{69298654-E280-9D4B-9717-7904FADC15B5}" name="phi" dataDxfId="13"/>
+    <tableColumn id="1" xr3:uid="{AF3C694B-2C8A-40EE-B8BB-2EC9EB81A87A}" name="mat_ID" dataDxfId="53"/>
+    <tableColumn id="2" xr3:uid="{B447FBC2-C455-4332-8F47-150B112A57E0}" name="name" dataDxfId="52"/>
+    <tableColumn id="3" xr3:uid="{BAFC6B47-7268-46CC-A881-892C9A1F4334}" name="strength_comp" dataDxfId="51"/>
+    <tableColumn id="4" xr3:uid="{6FC4C8EB-7581-4E67-81CE-C724161F0838}" name="strength_tens" dataDxfId="50"/>
+    <tableColumn id="5" xr3:uid="{A875970E-61A9-43B5-9361-7616A74C3147}" name="strength_bend" dataDxfId="49"/>
+    <tableColumn id="6" xr3:uid="{EF5B3A69-DD70-420A-88FF-4FE8772A2E14}" name="strength_shea" dataDxfId="48"/>
+    <tableColumn id="7" xr3:uid="{ED461A80-736C-42BD-81BC-C5C0C80FF34C}" name="E_modulus" dataDxfId="47"/>
+    <tableColumn id="8" xr3:uid="{68E47481-7028-4427-B126-2A046FC46737}" name="density_load" dataDxfId="46"/>
+    <tableColumn id="9" xr3:uid="{7AB34570-2BD4-417F-B141-70612577C7D6}" name="burn_rate" dataDxfId="45"/>
+    <tableColumn id="10" xr3:uid="{69298654-E280-9D4B-9717-7904FADC15B5}" name="phi" dataDxfId="44"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -8569,7 +8569,7 @@
                          T45&lt;=_xlfn.PERCENTILE.INC(_xlfn._xlws.FILTER($T$2:$T$148, ($L$2:$L$148=L45)*($W$2:$W$148=1)),0.9)
                ),1,0),
 0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z45" s="207">
         <f>2.01*Table2[[#This Row],[DENSITY]]</f>
@@ -9142,7 +9142,7 @@
                          T51&lt;=_xlfn.PERCENTILE.INC(_xlfn._xlws.FILTER($T$2:$T$148, ($L$2:$L$148=L51)*($W$2:$W$148=1)),0.9)
                ),1,0),
 0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z51" s="207">
         <f>2.01*Table2[[#This Row],[DENSITY]]</f>
@@ -9320,11 +9320,11 @@
       </c>
       <c r="W53" s="50">
         <f ca="1">IF(OR($D53="Ecoinvent",$D53="Betonsortenrechner",$D53="KBOB",$T53&lt;=0,Table2[[#This Row],[VALID_TO]]&lt;=TODAY()),0,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X53" s="198">
         <f ca="1">IF(Table2[[#This Row],[VALID_TO]]&gt;=TODAY(), 1, 0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y53" s="150" cm="1">
         <f t="array" aca="1" ref="Y53" ca="1">IF($W53&lt;&gt;0,
@@ -9415,11 +9415,11 @@
       </c>
       <c r="W54" s="50">
         <f ca="1">IF(OR($D54="Ecoinvent",$D54="Betonsortenrechner",$D54="KBOB",$T54&lt;=0,Table2[[#This Row],[VALID_TO]]&lt;=TODAY()),0,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X54" s="198">
         <f ca="1">IF(Table2[[#This Row],[VALID_TO]]&gt;=TODAY(), 1, 0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y54" s="150" cm="1">
         <f t="array" aca="1" ref="Y54" ca="1">IF($W54&lt;&gt;0,
@@ -13783,11 +13783,11 @@
       </c>
       <c r="W100" s="50">
         <f ca="1">IF(OR($D100="Ecoinvent",$D100="Betonsortenrechner",$D100="KBOB",$T100&lt;=0,Table2[[#This Row],[VALID_TO]]&lt;=TODAY()),0,1)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X100" s="198">
         <f ca="1">IF(Table2[[#This Row],[VALID_TO]]&gt;=TODAY(), 1, 0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y100" s="150" cm="1">
         <f t="array" aca="1" ref="Y100" ca="1">IF($W100&lt;&gt;0,
@@ -13796,7 +13796,7 @@
                          T100&lt;=_xlfn.PERCENTILE.INC(_xlfn._xlws.FILTER($T$2:$T$148, ($K$3:$K$149=K100)*($W$2:$W$148=1)),0.9)
                ),1,0),
 0)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z100" s="206">
         <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>

</xml_diff>

<commit_message>
Optimization of RC CS for upper reinforcement optimisation
</commit_message>
<xml_diff>
--- a/Database/260126_Datenbankdefinition.xlsx
+++ b/Database/260126_Datenbankdefinition.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jonathanbieg/Documents/Master Thesis/1_Code/Python Repository/SDSD_Bieg/Database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D943D0A5-A188-A14A-B5BD-62BE563A0ABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03CE3E68-0469-A74A-BDA0-BB8187620FEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17160" activeTab="1" xr2:uid="{58B6788A-438B-478E-898A-D53025B55ED1}"/>
   </bookViews>
@@ -16951,7 +16951,9 @@
       <c r="G5" s="56">
         <v>205000000000</v>
       </c>
-      <c r="H5" s="56"/>
+      <c r="H5" s="56">
+        <v>78500</v>
+      </c>
       <c r="I5" s="56"/>
       <c r="J5" s="56"/>
     </row>
@@ -17055,7 +17057,9 @@
       <c r="G9" s="211">
         <v>195000000000</v>
       </c>
-      <c r="H9" s="62"/>
+      <c r="H9" s="62">
+        <v>78500</v>
+      </c>
       <c r="I9" s="62"/>
       <c r="J9" s="62"/>
     </row>

</xml_diff>

<commit_message>
Saver before accustics implementation
</commit_message>
<xml_diff>
--- a/Database/260126_Datenbankdefinition.xlsx
+++ b/Database/260126_Datenbankdefinition.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jonathanbieg/Documents/Master Thesis/1_Code/Python Repository/SDSD_Bieg/Database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03CE3E68-0469-A74A-BDA0-BB8187620FEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1594CA47-2175-8149-86C5-8BB35061CC53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17160" activeTab="1" xr2:uid="{58B6788A-438B-478E-898A-D53025B55ED1}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17160" activeTab="2" xr2:uid="{58B6788A-438B-478E-898A-D53025B55ED1}"/>
   </bookViews>
   <sheets>
     <sheet name="products" sheetId="1" r:id="rId1"/>
@@ -93,7 +93,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1906" uniqueCount="525">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1904" uniqueCount="525">
   <si>
     <t>B500B</t>
   </si>
@@ -17177,11 +17177,11 @@
       <c r="B4" s="52" t="s">
         <v>402</v>
       </c>
-      <c r="C4" s="52" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="52" t="s">
-        <v>7</v>
+      <c r="C4" s="52">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="D4" s="52">
+        <v>6000</v>
       </c>
       <c r="E4" s="53">
         <v>80</v>

</xml_diff>

<commit_message>
Debugges Kser (TCC notches), Refined selfweight calculation (variation in concrete densities)
</commit_message>
<xml_diff>
--- a/Database/260126_Datenbankdefinition.xlsx
+++ b/Database/260126_Datenbankdefinition.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jonathanbieg/Documents/Master Thesis/1_Code/Python Repository/SDSD_Bieg/Database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3773198-9B14-1F43-8E20-3F9D5FEFC04D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB516A97-A7B2-5F49-9546-9C6F9CD423EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="660" windowWidth="29400" windowHeight="17160" xr2:uid="{58B6788A-438B-478E-898A-D53025B55ED1}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17160" activeTab="3" xr2:uid="{58B6788A-438B-478E-898A-D53025B55ED1}"/>
   </bookViews>
   <sheets>
     <sheet name="products" sheetId="1" r:id="rId1"/>
@@ -93,7 +93,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1904" uniqueCount="525">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1905" uniqueCount="526">
   <si>
     <t>B500B</t>
   </si>
@@ -1666,9 +1666,6 @@
     <t>phi</t>
   </si>
   <si>
-    <t>kerve</t>
-  </si>
-  <si>
     <t>K_ser</t>
   </si>
   <si>
@@ -1685,6 +1682,12 @@
   </si>
   <si>
     <t>Y1860</t>
+  </si>
+  <si>
+    <t>kerve_30</t>
+  </si>
+  <si>
+    <t>kerve_20</t>
   </si>
 </sst>
 </file>
@@ -1919,7 +1922,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="28">
+  <borders count="31">
     <border>
       <left/>
       <right/>
@@ -2232,12 +2235,49 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="hair">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="212">
+  <cellXfs count="221">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
@@ -2704,6 +2744,21 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="25" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="21" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="8" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4207,8 +4262,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1CD264FD-E2C0-E94F-B387-736226CC982D}" name="Tabelle42" displayName="Tabelle42" ref="A1:F6" totalsRowShown="0" headerRowDxfId="58" dataDxfId="56" headerRowBorderDxfId="57" tableBorderDxfId="55" totalsRowBorderDxfId="54">
-  <autoFilter ref="A1:F6" xr:uid="{1CD264FD-E2C0-E94F-B387-736226CC982D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1CD264FD-E2C0-E94F-B387-736226CC982D}" name="Tabelle42" displayName="Tabelle42" ref="A1:F7" totalsRowShown="0" headerRowDxfId="58" dataDxfId="56" headerRowBorderDxfId="57" tableBorderDxfId="55" totalsRowBorderDxfId="54">
+  <autoFilter ref="A1:F7" xr:uid="{1CD264FD-E2C0-E94F-B387-736226CC982D}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{6590463D-C242-4C4D-AA1F-6FA1F0D35E6F}" name="mat_ID" dataDxfId="53"/>
     <tableColumn id="2" xr3:uid="{603BAED4-55F2-D040-9D73-1611C1564A84}" name="name" dataDxfId="52"/>
@@ -4636,7 +4691,7 @@
         <v>497</v>
       </c>
       <c r="AC1" s="205" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="2" spans="1:29" s="10" customFormat="1" x14ac:dyDescent="0.2">
@@ -4727,7 +4782,7 @@
       <c r="AA2" s="11"/>
       <c r="AB2" s="21"/>
       <c r="AC2" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="3" spans="1:29" s="10" customFormat="1" x14ac:dyDescent="0.2">
@@ -4818,7 +4873,7 @@
       <c r="AA3" s="11"/>
       <c r="AB3" s="21"/>
       <c r="AC3" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="4" spans="1:29" s="10" customFormat="1" x14ac:dyDescent="0.2">
@@ -4909,7 +4964,7 @@
       <c r="AA4" s="11"/>
       <c r="AB4" s="21"/>
       <c r="AC4" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="5" spans="1:29" s="10" customFormat="1" x14ac:dyDescent="0.2">
@@ -5000,7 +5055,7 @@
       <c r="AA5" s="11"/>
       <c r="AB5" s="21"/>
       <c r="AC5" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="6" spans="1:29" s="10" customFormat="1" x14ac:dyDescent="0.2">
@@ -5091,7 +5146,7 @@
       <c r="AA6" s="11"/>
       <c r="AB6" s="21"/>
       <c r="AC6" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="7" spans="1:29" s="10" customFormat="1" x14ac:dyDescent="0.2">
@@ -5172,7 +5227,7 @@
       <c r="AA7" s="11"/>
       <c r="AB7" s="21"/>
       <c r="AC7" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="8" spans="1:29" s="10" customFormat="1" x14ac:dyDescent="0.2">
@@ -5253,7 +5308,7 @@
       <c r="AA8" s="11"/>
       <c r="AB8" s="21"/>
       <c r="AC8" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="9" spans="1:29" s="10" customFormat="1" x14ac:dyDescent="0.2">
@@ -5334,7 +5389,7 @@
       <c r="AA9" s="11"/>
       <c r="AB9" s="21"/>
       <c r="AC9" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="10" spans="1:29" s="10" customFormat="1" x14ac:dyDescent="0.2">
@@ -5415,7 +5470,7 @@
       <c r="AA10" s="11"/>
       <c r="AB10" s="21"/>
       <c r="AC10" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="11" spans="1:29" s="10" customFormat="1" x14ac:dyDescent="0.2">
@@ -5496,7 +5551,7 @@
       <c r="AA11" s="11"/>
       <c r="AB11" s="21"/>
       <c r="AC11" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="12" spans="1:29" s="10" customFormat="1" x14ac:dyDescent="0.2">
@@ -5587,7 +5642,7 @@
       <c r="AA12" s="11"/>
       <c r="AB12" s="21"/>
       <c r="AC12" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="13" spans="1:29" s="41" customFormat="1" x14ac:dyDescent="0.2">
@@ -5681,7 +5736,7 @@
       <c r="AA13" s="38"/>
       <c r="AB13" s="21"/>
       <c r="AC13" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="14" spans="1:29" s="41" customFormat="1" x14ac:dyDescent="0.2">
@@ -5775,7 +5830,7 @@
       <c r="AA14" s="38"/>
       <c r="AB14" s="21"/>
       <c r="AC14" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="15" spans="1:29" s="41" customFormat="1" x14ac:dyDescent="0.2">
@@ -5869,7 +5924,7 @@
       <c r="AA15" s="38"/>
       <c r="AB15" s="21"/>
       <c r="AC15" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="16" spans="1:29" s="41" customFormat="1" x14ac:dyDescent="0.2">
@@ -5963,7 +6018,7 @@
       <c r="AA16" s="38"/>
       <c r="AB16" s="21"/>
       <c r="AC16" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="17" spans="1:29" s="41" customFormat="1" x14ac:dyDescent="0.2">
@@ -6057,7 +6112,7 @@
       <c r="AA17" s="38"/>
       <c r="AB17" s="21"/>
       <c r="AC17" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="18" spans="1:29" s="41" customFormat="1" x14ac:dyDescent="0.2">
@@ -6151,7 +6206,7 @@
       <c r="AA18" s="38"/>
       <c r="AB18" s="21"/>
       <c r="AC18" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="19" spans="1:29" s="41" customFormat="1" x14ac:dyDescent="0.2">
@@ -6245,7 +6300,7 @@
       <c r="AA19" s="38"/>
       <c r="AB19" s="21"/>
       <c r="AC19" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="20" spans="1:29" s="41" customFormat="1" x14ac:dyDescent="0.2">
@@ -6339,7 +6394,7 @@
       <c r="AA20" s="38"/>
       <c r="AB20" s="21"/>
       <c r="AC20" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="21" spans="1:29" s="41" customFormat="1" x14ac:dyDescent="0.2">
@@ -6433,7 +6488,7 @@
       <c r="AA21" s="38"/>
       <c r="AB21" s="21"/>
       <c r="AC21" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="22" spans="1:29" s="41" customFormat="1" x14ac:dyDescent="0.2">
@@ -6527,7 +6582,7 @@
       <c r="AA22" s="38"/>
       <c r="AB22" s="21"/>
       <c r="AC22" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="23" spans="1:29" s="41" customFormat="1" x14ac:dyDescent="0.2">
@@ -6621,7 +6676,7 @@
       <c r="AA23" s="38"/>
       <c r="AB23" s="21"/>
       <c r="AC23" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="24" spans="1:29" x14ac:dyDescent="0.2">
@@ -6715,7 +6770,7 @@
       <c r="AA24" s="2"/>
       <c r="AB24" s="21"/>
       <c r="AC24" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="25" spans="1:29" x14ac:dyDescent="0.2">
@@ -6809,7 +6864,7 @@
       <c r="AA25" s="2"/>
       <c r="AB25" s="21"/>
       <c r="AC25" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="26" spans="1:29" x14ac:dyDescent="0.2">
@@ -6903,7 +6958,7 @@
       <c r="AA26" s="2"/>
       <c r="AB26" s="21"/>
       <c r="AC26" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="27" spans="1:29" x14ac:dyDescent="0.2">
@@ -6997,7 +7052,7 @@
       <c r="AA27" s="2"/>
       <c r="AB27" s="21"/>
       <c r="AC27" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="28" spans="1:29" x14ac:dyDescent="0.2">
@@ -7091,7 +7146,7 @@
       <c r="AA28" s="2"/>
       <c r="AB28" s="21"/>
       <c r="AC28" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="29" spans="1:29" x14ac:dyDescent="0.2">
@@ -7185,7 +7240,7 @@
       <c r="AA29" s="2"/>
       <c r="AB29" s="21"/>
       <c r="AC29" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="30" spans="1:29" x14ac:dyDescent="0.2">
@@ -7279,7 +7334,7 @@
       <c r="AA30" s="2"/>
       <c r="AB30" s="21"/>
       <c r="AC30" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="31" spans="1:29" x14ac:dyDescent="0.2">
@@ -7355,7 +7410,7 @@
       <c r="AA31" s="2"/>
       <c r="AB31" s="179"/>
       <c r="AC31" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="32" spans="1:29" x14ac:dyDescent="0.2">
@@ -7431,7 +7486,7 @@
       <c r="AA32" s="2"/>
       <c r="AB32" s="182"/>
       <c r="AC32" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="33" spans="1:29" x14ac:dyDescent="0.2">
@@ -7507,7 +7562,7 @@
       <c r="AA33" s="2"/>
       <c r="AB33" s="182"/>
       <c r="AC33" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="34" spans="1:29" x14ac:dyDescent="0.2">
@@ -7583,7 +7638,7 @@
       <c r="AA34" s="2"/>
       <c r="AB34" s="182"/>
       <c r="AC34" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="35" spans="1:29" x14ac:dyDescent="0.2">
@@ -7659,7 +7714,7 @@
       <c r="AA35" s="2"/>
       <c r="AB35" s="182"/>
       <c r="AC35" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="36" spans="1:29" x14ac:dyDescent="0.2">
@@ -7735,7 +7790,7 @@
       <c r="AA36" s="2"/>
       <c r="AB36" s="182"/>
       <c r="AC36" s="210">
-        <v>0.55000000000000004</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="37" spans="1:29" s="15" customFormat="1" ht="16" thickBot="1" x14ac:dyDescent="0.25">
@@ -7800,7 +7855,7 @@
       <c r="V37" s="142">
         <v>13</v>
       </c>
-      <c r="W37" s="50">
+      <c r="W37" s="212">
         <f ca="1">IF(OR($D37="Ecoinvent",$D37="Betonsortenrechner",$D37="KBOB",$T37&lt;=0,Table2[[#This Row],[VALID_TO]]&lt;=TODAY()),0,1)</f>
         <v>0</v>
       </c>
@@ -7817,13 +7872,13 @@
 0)</f>
         <v>0</v>
       </c>
-      <c r="Z37" s="206">
+      <c r="Z37" s="213">
         <v>206</v>
       </c>
       <c r="AA37" s="13"/>
-      <c r="AB37" s="182"/>
-      <c r="AC37" s="210">
-        <v>0.55000000000000004</v>
+      <c r="AB37" s="214"/>
+      <c r="AC37" s="215">
+        <v>0.4</v>
       </c>
     </row>
     <row r="38" spans="1:29" s="15" customFormat="1" x14ac:dyDescent="0.2">
@@ -9511,7 +9566,7 @@
       <c r="V55" s="144" t="s">
         <v>167</v>
       </c>
-      <c r="W55" s="50">
+      <c r="W55" s="212">
         <f ca="1">IF(OR($D55="Ecoinvent",$D55="Betonsortenrechner",$D55="KBOB",$T55&lt;=0,Table2[[#This Row],[VALID_TO]]&lt;=TODAY()),0,1)</f>
         <v>0</v>
       </c>
@@ -9528,13 +9583,13 @@
 0)</f>
         <v>0</v>
       </c>
-      <c r="Z55" s="207">
+      <c r="Z55" s="216">
         <f>2.01*Table2[[#This Row],[DENSITY]]</f>
         <v>15778.499999999998</v>
       </c>
       <c r="AA55" s="4"/>
-      <c r="AB55" s="183"/>
-      <c r="AC55" s="210">
+      <c r="AB55" s="217"/>
+      <c r="AC55" s="215">
         <f>0.009*Table2[[#This Row],[DENSITY]]</f>
         <v>70.649999999999991</v>
       </c>
@@ -9624,8 +9679,8 @@
         <v>0</v>
       </c>
       <c r="Z56" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA56" s="11"/>
       <c r="AB56" s="183"/>
@@ -9718,8 +9773,8 @@
         <v>0</v>
       </c>
       <c r="Z57" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA57" s="11"/>
       <c r="AB57" s="183"/>
@@ -9812,8 +9867,8 @@
         <v>0</v>
       </c>
       <c r="Z58" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA58" s="11"/>
       <c r="AB58" s="183"/>
@@ -9906,8 +9961,8 @@
         <v>0</v>
       </c>
       <c r="Z59" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA59" s="11"/>
       <c r="AB59" s="183"/>
@@ -10000,8 +10055,8 @@
         <v>0</v>
       </c>
       <c r="Z60" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>1700</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1250</v>
       </c>
       <c r="AA60" s="11"/>
       <c r="AB60" s="183"/>
@@ -10094,8 +10149,8 @@
         <v>0</v>
       </c>
       <c r="Z61" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>1700</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1250</v>
       </c>
       <c r="AA61" s="11"/>
       <c r="AB61" s="183"/>
@@ -10185,8 +10240,8 @@
         <v>0</v>
       </c>
       <c r="Z62" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA62" s="16"/>
       <c r="AB62" s="182"/>
@@ -10273,8 +10328,8 @@
         <v>0</v>
       </c>
       <c r="Z63" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA63" s="16"/>
       <c r="AB63" s="182"/>
@@ -10363,8 +10418,8 @@
         <v>0</v>
       </c>
       <c r="Z64" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA64" s="16"/>
       <c r="AB64" s="182"/>
@@ -10451,8 +10506,8 @@
         <v>0</v>
       </c>
       <c r="Z65" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA65" s="16"/>
       <c r="AB65" s="182"/>
@@ -10539,8 +10594,8 @@
         <v>0</v>
       </c>
       <c r="Z66" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>1700</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1250</v>
       </c>
       <c r="AA66" s="16"/>
       <c r="AB66" s="182"/>
@@ -10634,8 +10689,8 @@
         <v>0</v>
       </c>
       <c r="Z67" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA67" s="2" t="s">
         <v>428</v>
@@ -10731,8 +10786,8 @@
         <v>1</v>
       </c>
       <c r="Z68" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA68" s="2" t="s">
         <v>429</v>
@@ -10828,8 +10883,8 @@
         <v>0</v>
       </c>
       <c r="Z69" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA69" s="2"/>
       <c r="AB69" s="21"/>
@@ -10923,8 +10978,8 @@
         <v>1</v>
       </c>
       <c r="Z70" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA70" s="2" t="s">
         <v>431</v>
@@ -11020,8 +11075,8 @@
         <v>1</v>
       </c>
       <c r="Z71" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA71" s="2" t="s">
         <v>430</v>
@@ -11117,8 +11172,8 @@
         <v>1</v>
       </c>
       <c r="Z72" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA72" s="2" t="s">
         <v>431</v>
@@ -11214,8 +11269,8 @@
         <v>0</v>
       </c>
       <c r="Z73" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA73" s="2"/>
       <c r="AB73" s="21"/>
@@ -11309,8 +11364,8 @@
         <v>1</v>
       </c>
       <c r="Z74" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>1700</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1250</v>
       </c>
       <c r="AA74" s="63" t="s">
         <v>416</v>
@@ -11408,8 +11463,8 @@
         <v>0</v>
       </c>
       <c r="Z75" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA75" s="2" t="s">
         <v>433</v>
@@ -11505,8 +11560,8 @@
         <v>0</v>
       </c>
       <c r="Z76" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA76" s="2" t="s">
         <v>433</v>
@@ -11601,8 +11656,8 @@
         <v>0</v>
       </c>
       <c r="Z77" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA77" s="2"/>
       <c r="AB77" s="21"/>
@@ -11696,8 +11751,8 @@
         <v>1</v>
       </c>
       <c r="Z78" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA78" s="2"/>
       <c r="AB78" s="21"/>
@@ -11791,8 +11846,8 @@
         <v>0</v>
       </c>
       <c r="Z79" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA79" s="2" t="s">
         <v>438</v>
@@ -11888,8 +11943,8 @@
         <v>0</v>
       </c>
       <c r="Z80" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA80" s="2" t="s">
         <v>439</v>
@@ -11985,8 +12040,8 @@
         <v>1</v>
       </c>
       <c r="Z81" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA81" s="2" t="s">
         <v>440</v>
@@ -12084,8 +12139,8 @@
         <v>0</v>
       </c>
       <c r="Z82" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA82" s="2"/>
       <c r="AB82" s="21"/>
@@ -12179,8 +12234,8 @@
         <v>1</v>
       </c>
       <c r="Z83" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA83" s="2"/>
       <c r="AB83" s="21"/>
@@ -12274,8 +12329,8 @@
         <v>1</v>
       </c>
       <c r="Z84" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA84" s="2"/>
       <c r="AB84" s="21"/>
@@ -12361,8 +12416,8 @@
         <v>0</v>
       </c>
       <c r="Z85" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA85" s="2"/>
       <c r="AB85" s="21"/>
@@ -12456,8 +12511,8 @@
         <v>0</v>
       </c>
       <c r="Z86" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA86" s="2"/>
       <c r="AB86" s="21"/>
@@ -12548,8 +12603,8 @@
         <v>0</v>
       </c>
       <c r="Z87" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA87" s="2"/>
       <c r="AB87" s="21"/>
@@ -12643,8 +12698,8 @@
         <v>1</v>
       </c>
       <c r="Z88" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA88" s="2"/>
       <c r="AB88" s="21"/>
@@ -12738,8 +12793,8 @@
         <v>1</v>
       </c>
       <c r="Z89" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA89" s="2" t="s">
         <v>434</v>
@@ -12834,8 +12889,8 @@
         <v>0</v>
       </c>
       <c r="Z90" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA90" s="2" t="s">
         <v>432</v>
@@ -12931,8 +12986,8 @@
         <v>1</v>
       </c>
       <c r="Z91" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA91" s="2" t="s">
         <v>435</v>
@@ -13028,8 +13083,8 @@
         <v>1</v>
       </c>
       <c r="Z92" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA92" s="2" t="s">
         <v>437</v>
@@ -13127,8 +13182,8 @@
         <v>1</v>
       </c>
       <c r="Z93" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA93" s="2" t="s">
         <v>434</v>
@@ -13224,8 +13279,8 @@
         <v>0</v>
       </c>
       <c r="Z94" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA94" s="2"/>
       <c r="AB94" s="21"/>
@@ -13319,8 +13374,8 @@
         <v>0</v>
       </c>
       <c r="Z95" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA95" s="2"/>
       <c r="AB95" s="21"/>
@@ -13414,8 +13469,8 @@
         <v>0</v>
       </c>
       <c r="Z96" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA96" s="2" t="s">
         <v>438</v>
@@ -13511,8 +13566,8 @@
         <v>0</v>
       </c>
       <c r="Z97" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>1700</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1250</v>
       </c>
       <c r="AA97" s="2" t="s">
         <v>418</v>
@@ -13608,8 +13663,8 @@
         <v>0</v>
       </c>
       <c r="Z98" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>1700</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1250</v>
       </c>
       <c r="AA98" s="2" t="s">
         <v>417</v>
@@ -13705,8 +13760,8 @@
         <v>0</v>
       </c>
       <c r="Z99" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>1700</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1250</v>
       </c>
       <c r="AA99" s="2" t="s">
         <v>420</v>
@@ -13802,8 +13857,8 @@
         <v>0</v>
       </c>
       <c r="Z100" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>1700</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1250</v>
       </c>
       <c r="AA100" s="2" t="s">
         <v>421</v>
@@ -13899,8 +13954,8 @@
         <v>0</v>
       </c>
       <c r="Z101" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>1700</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1250</v>
       </c>
       <c r="AA101" s="2" t="s">
         <v>422</v>
@@ -13980,7 +14035,7 @@
         <f>(0.341+6.93+800)/Table2[[#This Row],[DENSITY]]*1000</f>
         <v>1543.5391969407265</v>
       </c>
-      <c r="W102" s="50">
+      <c r="W102" s="218">
         <f ca="1">IF(OR($D102="Ecoinvent",$D102="Betonsortenrechner",$D102="KBOB",$T102&lt;=0,Table2[[#This Row],[VALID_TO]]&lt;=TODAY()),0,1)</f>
         <v>1</v>
       </c>
@@ -13998,8 +14053,8 @@
         <v>0</v>
       </c>
       <c r="Z102" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>1700</v>
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1250</v>
       </c>
       <c r="AA102" s="2" t="s">
         <v>426</v>
@@ -14079,11 +14134,11 @@
         <f>(0.8+4.9+758)/Table2[[#This Row],[DENSITY]]*1000</f>
         <v>1631.8376068376069</v>
       </c>
-      <c r="W103" s="50">
+      <c r="W103" s="212">
         <f ca="1">IF(OR($D103="Ecoinvent",$D103="Betonsortenrechner",$D103="KBOB",$T103&lt;=0,Table2[[#This Row],[VALID_TO]]&lt;=TODAY()),0,1)</f>
         <v>0</v>
       </c>
-      <c r="X103" s="198">
+      <c r="X103" s="199">
         <f ca="1">IF(Table2[[#This Row],[VALID_TO]]&gt;=TODAY(), 1, 0)</f>
         <v>0</v>
       </c>
@@ -14096,15 +14151,15 @@
 0)</f>
         <v>0</v>
       </c>
-      <c r="Z103" s="206">
-        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1700,2200)</f>
-        <v>2200</v>
+      <c r="Z103" s="213">
+        <f>IF(Table2[[#This Row],[MATERIAL]]="Solid_structural_timber",1250,1750)</f>
+        <v>1750</v>
       </c>
       <c r="AA103" s="4" t="s">
         <v>467</v>
       </c>
       <c r="AB103" s="37"/>
-      <c r="AC103" s="210">
+      <c r="AC103" s="215">
         <v>1</v>
       </c>
     </row>
@@ -15497,7 +15552,7 @@
         <f>1.1+9.68+26.7</f>
         <v>37.479999999999997</v>
       </c>
-      <c r="W118" s="158">
+      <c r="W118" s="219">
         <v>0</v>
       </c>
       <c r="X118" s="193">
@@ -15591,7 +15646,7 @@
         <f>21.5+68.6</f>
         <v>90.1</v>
       </c>
-      <c r="W119" s="50">
+      <c r="W119" s="218">
         <f ca="1">IF(OR($D119="Ecoinvent",$D119="Betonsortenrechner",$D119="KBOB",$T119&lt;=0,Table2[[#This Row],[VALID_TO]]&lt;=TODAY()),0,1)</f>
         <v>0</v>
       </c>
@@ -15686,7 +15741,7 @@
         <f>5.85+7.57</f>
         <v>13.42</v>
       </c>
-      <c r="W120" s="50">
+      <c r="W120" s="218">
         <f ca="1">IF(OR($D120="Ecoinvent",$D120="Betonsortenrechner",$D120="KBOB",$T120&lt;=0,Table2[[#This Row],[VALID_TO]]&lt;=TODAY()),0,1)</f>
         <v>1</v>
       </c>
@@ -15782,7 +15837,7 @@
         <f>21.4+6.84+2.22</f>
         <v>30.459999999999997</v>
       </c>
-      <c r="W121" s="50">
+      <c r="W121" s="212">
         <f ca="1">IF(OR($D121="Ecoinvent",$D121="Betonsortenrechner",$D121="KBOB",$T121&lt;=0,Table2[[#This Row],[VALID_TO]]&lt;=TODAY()),0,1)</f>
         <v>0</v>
       </c>
@@ -15799,7 +15854,7 @@
 0)</f>
         <v>0</v>
       </c>
-      <c r="Z121" s="208">
+      <c r="Z121" s="216">
         <f>17*Table2[[#This Row],[DENSITY]]</f>
         <v>133450</v>
       </c>
@@ -15807,7 +15862,7 @@
         <v>493</v>
       </c>
       <c r="AB121" s="37"/>
-      <c r="AC121" s="210">
+      <c r="AC121" s="215">
         <f t="shared" ref="AC121" si="2">1.2</f>
         <v>1.2</v>
       </c>
@@ -15851,7 +15906,7 @@
         <v>427</v>
       </c>
       <c r="N122" s="26" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="O122" s="26"/>
       <c r="P122" s="3"/>
@@ -15938,7 +15993,7 @@
         <v>427</v>
       </c>
       <c r="N123" s="26" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="O123" s="26"/>
       <c r="P123" s="3"/>
@@ -16023,7 +16078,7 @@
         <v>427</v>
       </c>
       <c r="N124" s="26" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="O124" s="26"/>
       <c r="P124" s="3"/>
@@ -16110,7 +16165,7 @@
         <v>427</v>
       </c>
       <c r="N125" s="26" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="O125" s="26"/>
       <c r="P125" s="3"/>
@@ -16198,7 +16253,7 @@
         <v>427</v>
       </c>
       <c r="N126" s="26" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="O126" s="26"/>
       <c r="P126" s="3"/>
@@ -16284,7 +16339,7 @@
         <v>427</v>
       </c>
       <c r="N127" s="26" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="O127" s="26"/>
       <c r="P127" s="3"/>
@@ -16368,7 +16423,7 @@
         <v>427</v>
       </c>
       <c r="N128" s="26" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="O128" s="26"/>
       <c r="P128" s="3"/>
@@ -16453,7 +16508,7 @@
         <v>427</v>
       </c>
       <c r="N129" s="26" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="O129" s="26"/>
       <c r="P129" s="3"/>
@@ -16538,7 +16593,7 @@
         <v>427</v>
       </c>
       <c r="N130" s="29" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="O130" s="29"/>
       <c r="P130" s="5"/>
@@ -16556,7 +16611,7 @@
         <f>3.59+0.0792+0.326</f>
         <v>3.9952000000000001</v>
       </c>
-      <c r="W130" s="50">
+      <c r="W130" s="212">
         <f ca="1">IF(OR($D130="Ecoinvent",$D130="Betonsortenrechner",$D130="KBOB",$T130&lt;=0,Table2[[#This Row],[VALID_TO]]&lt;=TODAY()),0,1)</f>
         <v>1</v>
       </c>
@@ -16573,13 +16628,13 @@
 0)</f>
         <v>0</v>
       </c>
-      <c r="Z130" s="209">
+      <c r="Z130" s="220">
         <f t="shared" si="3"/>
         <v>78500</v>
       </c>
       <c r="AA130" s="4"/>
-      <c r="AB130" s="21"/>
-      <c r="AC130" s="210">
+      <c r="AB130" s="37"/>
+      <c r="AC130" s="215">
         <f t="shared" si="4"/>
         <v>157</v>
       </c>
@@ -17049,7 +17104,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="62" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="C9" s="62"/>
       <c r="D9" s="62">
@@ -17113,10 +17168,10 @@
         <v>399</v>
       </c>
       <c r="H1" s="204" t="s">
+        <v>520</v>
+      </c>
+      <c r="I1" s="204" t="s">
         <v>521</v>
-      </c>
-      <c r="I1" s="204" t="s">
-        <v>522</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
@@ -17145,7 +17200,7 @@
         <v>9626</v>
       </c>
       <c r="I2">
-        <v>0.55000000000000004</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
@@ -17172,7 +17227,7 @@
         <v>391</v>
       </c>
       <c r="I3">
-        <v>0.55000000000000004</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
@@ -17200,7 +17255,7 @@
         <v>335</v>
       </c>
       <c r="I4">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
@@ -17253,7 +17308,7 @@
         <v>335</v>
       </c>
       <c r="I6">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
@@ -17279,7 +17334,7 @@
         <v>335</v>
       </c>
       <c r="I7">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>
@@ -17298,6 +17353,7 @@
     <col min="2" max="2" width="11.1640625" customWidth="1"/>
     <col min="3" max="3" width="27.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="27.33203125" customWidth="1"/>
+    <col min="6" max="7" width="12.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -17308,16 +17364,16 @@
         <v>407</v>
       </c>
       <c r="C1" s="61" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="D1" s="61" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="E1" s="61" t="s">
         <v>127</v>
       </c>
       <c r="F1" s="61" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -17334,10 +17390,10 @@
         <v>5830000</v>
       </c>
       <c r="E2" s="203">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F2" s="203">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -17354,10 +17410,10 @@
         <v>7780000</v>
       </c>
       <c r="E3" s="56">
-        <v>9</v>
+        <v>5.5</v>
       </c>
       <c r="F3" s="56">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -17374,10 +17430,10 @@
         <v>9700000</v>
       </c>
       <c r="E4" s="56">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F4" s="56">
-        <v>2.5000000000000001E-2</v>
+        <v>1.4999999999999999E-2</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -17394,10 +17450,10 @@
         <v>11670000</v>
       </c>
       <c r="E5" s="56">
-        <v>11</v>
+        <v>6.5</v>
       </c>
       <c r="F5" s="56">
-        <v>2.5000000000000001E-2</v>
+        <v>1.4999999999999999E-2</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -17405,7 +17461,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="56" t="s">
-        <v>518</v>
+        <v>525</v>
       </c>
       <c r="C6" s="56"/>
       <c r="D6" s="56">
@@ -17415,6 +17471,25 @@
         <v>30</v>
       </c>
       <c r="F6" s="62">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" s="62">
+        <v>6</v>
+      </c>
+      <c r="B7" s="62" t="s">
+        <v>524</v>
+      </c>
+      <c r="C7" s="62"/>
+      <c r="D7" s="62">
+        <f>D6*1.5</f>
+        <v>1500000000</v>
+      </c>
+      <c r="E7" s="62">
+        <v>30</v>
+      </c>
+      <c r="F7" s="62">
         <v>0.01</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adjusted plots for Latex Document
</commit_message>
<xml_diff>
--- a/Database/260126_Datenbankdefinition.xlsx
+++ b/Database/260126_Datenbankdefinition.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jonathanbieg/Documents/Master Thesis/1_Code/Python Repository/SDSD_Bieg/Database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB516A97-A7B2-5F49-9546-9C6F9CD423EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08A7B295-EF35-F44C-9023-62AF7636D597}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17160" activeTab="3" xr2:uid="{58B6788A-438B-478E-898A-D53025B55ED1}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17160" xr2:uid="{58B6788A-438B-478E-898A-D53025B55ED1}"/>
   </bookViews>
   <sheets>
     <sheet name="products" sheetId="1" r:id="rId1"/>
@@ -2277,7 +2277,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="221">
+  <cellXfs count="224">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
@@ -2759,6 +2759,15 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5188,7 +5197,9 @@
       <c r="N7" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="O7" s="25"/>
+      <c r="O7" s="221">
+        <v>2400</v>
+      </c>
       <c r="P7" s="12" t="s">
         <v>167</v>
       </c>
@@ -5269,7 +5280,9 @@
       <c r="N8" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="O8" s="25"/>
+      <c r="O8" s="221">
+        <v>2400</v>
+      </c>
       <c r="P8" s="12" t="s">
         <v>167</v>
       </c>
@@ -5350,7 +5363,9 @@
       <c r="N9" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="O9" s="25"/>
+      <c r="O9" s="221">
+        <v>2400</v>
+      </c>
       <c r="P9" s="12" t="s">
         <v>167</v>
       </c>
@@ -5431,7 +5446,9 @@
       <c r="N10" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="O10" s="25"/>
+      <c r="O10" s="221">
+        <v>2400</v>
+      </c>
       <c r="P10" s="12" t="s">
         <v>167</v>
       </c>
@@ -5512,7 +5529,9 @@
       <c r="N11" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="O11" s="25"/>
+      <c r="O11" s="221">
+        <v>2400</v>
+      </c>
       <c r="P11" s="12" t="s">
         <v>167</v>
       </c>
@@ -15908,7 +15927,9 @@
       <c r="N122" s="26" t="s">
         <v>523</v>
       </c>
-      <c r="O122" s="26"/>
+      <c r="O122" s="222">
+        <v>7850</v>
+      </c>
       <c r="P122" s="3"/>
       <c r="Q122" s="3"/>
       <c r="R122" s="3"/>
@@ -15995,7 +16016,9 @@
       <c r="N123" s="26" t="s">
         <v>523</v>
       </c>
-      <c r="O123" s="26"/>
+      <c r="O123" s="222">
+        <v>7850</v>
+      </c>
       <c r="P123" s="3"/>
       <c r="Q123" s="3"/>
       <c r="R123" s="3"/>
@@ -16080,7 +16103,9 @@
       <c r="N124" s="26" t="s">
         <v>523</v>
       </c>
-      <c r="O124" s="26"/>
+      <c r="O124" s="222">
+        <v>7850</v>
+      </c>
       <c r="P124" s="3"/>
       <c r="Q124" s="3"/>
       <c r="R124" s="3"/>
@@ -16167,7 +16192,9 @@
       <c r="N125" s="26" t="s">
         <v>523</v>
       </c>
-      <c r="O125" s="26"/>
+      <c r="O125" s="222">
+        <v>7850</v>
+      </c>
       <c r="P125" s="3"/>
       <c r="Q125" s="3"/>
       <c r="R125" s="3"/>
@@ -16255,7 +16282,9 @@
       <c r="N126" s="26" t="s">
         <v>523</v>
       </c>
-      <c r="O126" s="26"/>
+      <c r="O126" s="222">
+        <v>7850</v>
+      </c>
       <c r="P126" s="3"/>
       <c r="Q126" s="3"/>
       <c r="R126" s="3"/>
@@ -16341,7 +16370,9 @@
       <c r="N127" s="26" t="s">
         <v>523</v>
       </c>
-      <c r="O127" s="26"/>
+      <c r="O127" s="222">
+        <v>7850</v>
+      </c>
       <c r="P127" s="3"/>
       <c r="Q127" s="3"/>
       <c r="R127" s="3"/>
@@ -16425,7 +16456,9 @@
       <c r="N128" s="26" t="s">
         <v>523</v>
       </c>
-      <c r="O128" s="26"/>
+      <c r="O128" s="222">
+        <v>7850</v>
+      </c>
       <c r="P128" s="3"/>
       <c r="Q128" s="3"/>
       <c r="R128" s="3"/>
@@ -16510,7 +16543,9 @@
       <c r="N129" s="26" t="s">
         <v>523</v>
       </c>
-      <c r="O129" s="26"/>
+      <c r="O129" s="222">
+        <v>7850</v>
+      </c>
       <c r="P129" s="3"/>
       <c r="Q129" s="3"/>
       <c r="R129" s="3"/>
@@ -16595,7 +16630,9 @@
       <c r="N130" s="29" t="s">
         <v>523</v>
       </c>
-      <c r="O130" s="29"/>
+      <c r="O130" s="223">
+        <v>7850</v>
+      </c>
       <c r="P130" s="5"/>
       <c r="Q130" s="5"/>
       <c r="R130" s="5"/>

</xml_diff>